<commit_message>
feat: implement product review scanner and integrate 2-day buffer window filtering
</commit_message>
<xml_diff>
--- a/reports/telegram_sebi_10day_report.xlsx
+++ b/reports/telegram_sebi_10day_report.xlsx
@@ -624,10 +624,10 @@
         <v>569271</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>9101769</v>
+        <v>9566819</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -720,10 +720,10 @@
         <v>495829</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1649023</v>
+        <v>2640681</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -816,10 +816,10 @@
         <v>393135</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1134968</v>
+        <v>1170328</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -1008,10 +1008,10 @@
         <v>211523</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1302587</v>
+        <v>1396959</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -1104,10 +1104,10 @@
         <v>162819</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>2701443</v>
+        <v>2949773</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -1200,10 +1200,10 @@
         <v>158965</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>917558</v>
+        <v>979764</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -1296,10 +1296,10 @@
         <v>151478</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1934880</v>
+        <v>2131254</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1584,10 +1584,10 @@
         <v>131492</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1731625</v>
+        <v>1969403</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1680,10 +1680,10 @@
         <v>127846</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1310920</v>
+        <v>1335072</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1776,10 +1776,10 @@
         <v>114194</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>736088</v>
+        <v>752302</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1872,10 +1872,10 @@
         <v>107479</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1034652</v>
+        <v>1249610</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -2256,10 +2256,10 @@
         <v>99486</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>1527265</v>
+        <v>1576759</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -2448,10 +2448,10 @@
         <v>94169</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1450780</v>
+        <v>1639118</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
@@ -2640,10 +2640,10 @@
         <v>88046</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>892572</v>
+        <v>1037940</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -2832,10 +2832,10 @@
         <v>85649</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>373966</v>
+        <v>544740</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -2928,10 +2928,10 @@
         <v>82493</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>85915</v>
+        <v>250901</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -3024,10 +3024,10 @@
         <v>80760</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>730180</v>
+        <v>737380</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -3120,10 +3120,10 @@
         <v>80739</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1029889</v>
+        <v>1048937</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -3216,10 +3216,10 @@
         <v>79502</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>629900</v>
+        <v>654362</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -3312,10 +3312,10 @@
         <v>76419</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>911091</v>
+        <v>955037</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -3408,10 +3408,10 @@
         <v>75133</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>423439</v>
+        <v>511025</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
@@ -3600,10 +3600,10 @@
         <v>69504</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>626629</v>
+        <v>688147</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
@@ -3696,10 +3696,10 @@
         <v>69387</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>284308</v>
+        <v>423082</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -3792,10 +3792,10 @@
         <v>68460</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>305610</v>
+        <v>310460</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -3888,10 +3888,10 @@
         <v>68202</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>343336</v>
+        <v>419510</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -3984,10 +3984,10 @@
         <v>66718</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>624565</v>
+        <v>758001</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
@@ -4080,10 +4080,10 @@
         <v>66703</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>419009</v>
+        <v>468417</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -4176,10 +4176,10 @@
         <v>65193</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>703134</v>
+        <v>712488</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -4272,10 +4272,10 @@
         <v>65111</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>769272</v>
+        <v>793388</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -4464,10 +4464,10 @@
         <v>59566</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>654953</v>
+        <v>660847</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -4560,10 +4560,10 @@
         <v>58582</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>692189</v>
+        <v>780429</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -4656,10 +4656,10 @@
         <v>58176</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>418679</v>
+        <v>531169</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -4848,10 +4848,10 @@
         <v>57276</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>349151</v>
+        <v>427557</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -4944,10 +4944,10 @@
         <v>55945</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>529276</v>
+        <v>535862</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -5040,10 +5040,10 @@
         <v>55901</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>164908</v>
+        <v>271120</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -5136,10 +5136,10 @@
         <v>55249</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>205191</v>
+        <v>315689</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
@@ -5232,10 +5232,10 @@
         <v>54993</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>591885</v>
+        <v>636089</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -5328,10 +5328,10 @@
         <v>54825</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>588209</v>
+        <v>633831</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -5424,10 +5424,10 @@
         <v>53890</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>965798</v>
+        <v>1072942</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -5712,10 +5712,10 @@
         <v>51138</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>377082</v>
+        <v>479358</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -6000,10 +6000,10 @@
         <v>49470</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>497343</v>
+        <v>587903</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
@@ -6096,10 +6096,10 @@
         <v>48785</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>783292</v>
+        <v>843794</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
@@ -6192,10 +6192,10 @@
         <v>48520</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>470865</v>
+        <v>567905</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
@@ -6384,10 +6384,10 @@
         <v>48086</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>689650</v>
+        <v>728212</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
@@ -6480,10 +6480,10 @@
         <v>47899</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>138089</v>
+        <v>233887</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
@@ -6576,10 +6576,10 @@
         <v>47876</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>605490</v>
+        <v>639796</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
@@ -6672,10 +6672,10 @@
         <v>46941</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>417553</v>
+        <v>478081</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -6864,10 +6864,10 @@
         <v>43995</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>576062</v>
+        <v>634898</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
@@ -6960,10 +6960,10 @@
         <v>43416</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>127531</v>
+        <v>130149</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
@@ -7056,10 +7056,10 @@
         <v>43047</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>476375</v>
+        <v>510743</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
@@ -7344,10 +7344,10 @@
         <v>41300</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>148518</v>
+        <v>162268</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
@@ -7440,10 +7440,10 @@
         <v>41270</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>161190</v>
+        <v>171372</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
@@ -7536,10 +7536,10 @@
         <v>40719</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>592081</v>
+        <v>620479</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
@@ -7728,10 +7728,10 @@
         <v>39288</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>498197</v>
+        <v>525849</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
@@ -7824,10 +7824,10 @@
         <v>39193</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>146918</v>
+        <v>166428</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
@@ -8016,10 +8016,10 @@
         <v>38479</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>614108</v>
+        <v>672596</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
@@ -8208,10 +8208,10 @@
         <v>37702</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>106253</v>
+        <v>181657</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
@@ -8496,10 +8496,10 @@
         <v>37246</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>198941</v>
+        <v>210781</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
@@ -8688,10 +8688,10 @@
         <v>36417</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>328781</v>
+        <v>371127</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
@@ -8784,10 +8784,10 @@
         <v>35954</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>50860</v>
+        <v>122768</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
@@ -8880,10 +8880,10 @@
         <v>35835</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>416402</v>
+        <v>479584</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
@@ -8976,10 +8976,10 @@
         <v>35080</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>351590</v>
+        <v>421750</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
@@ -9072,10 +9072,10 @@
         <v>34616</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>72466</v>
+        <v>87864</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -9168,10 +9168,10 @@
         <v>34370</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>462886</v>
+        <v>508898</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
@@ -9264,10 +9264,10 @@
         <v>34334</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>338598</v>
+        <v>356670</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
@@ -9360,10 +9360,10 @@
         <v>33783</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>465470</v>
+        <v>476782</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
@@ -9456,10 +9456,10 @@
         <v>33544</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>506777</v>
+        <v>525945</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -9552,10 +9552,10 @@
         <v>33294</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>193953</v>
+        <v>209103</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
@@ -9648,10 +9648,10 @@
         <v>33238</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>136549</v>
+        <v>161505</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
@@ -9744,10 +9744,10 @@
         <v>33063</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>435281</v>
+        <v>484863</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
@@ -9840,10 +9840,10 @@
         <v>32476</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>184120</v>
+        <v>218646</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
@@ -9936,10 +9936,10 @@
         <v>32351</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>205287</v>
+        <v>220907</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
@@ -10032,10 +10032,10 @@
         <v>31814</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>401606</v>
+        <v>440426</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K100" s="2" t="inlineStr">
         <is>
@@ -10128,10 +10128,10 @@
         <v>31499</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>227203</v>
+        <v>240623</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
@@ -10224,10 +10224,10 @@
         <v>31199</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>277460</v>
+        <v>315874</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
@@ -10320,10 +10320,10 @@
         <v>30867</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>69687</v>
+        <v>131421</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
@@ -10416,10 +10416,10 @@
         <v>30716</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>260460</v>
+        <v>272106</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
@@ -10512,10 +10512,10 @@
         <v>30200</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>69338</v>
+        <v>87214</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
@@ -10704,10 +10704,10 @@
         <v>29237</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>359942</v>
+        <v>369528</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
@@ -10800,10 +10800,10 @@
         <v>29222</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>256313</v>
+        <v>281041</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
@@ -10992,10 +10992,10 @@
         <v>28689</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>258780</v>
+        <v>278060</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
@@ -11184,10 +11184,10 @@
         <v>28316</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>204788</v>
+        <v>220410</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
@@ -11280,10 +11280,10 @@
         <v>28151</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>125077</v>
+        <v>174457</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
@@ -11376,10 +11376,10 @@
         <v>27761</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>246267</v>
+        <v>301789</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
@@ -11664,10 +11664,10 @@
         <v>27646</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>239265</v>
+        <v>251679</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K117" s="2" t="inlineStr">
         <is>
@@ -11760,10 +11760,10 @@
         <v>27571</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>193281</v>
+        <v>215865</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K118" s="2" t="inlineStr">
         <is>
@@ -11856,10 +11856,10 @@
         <v>27501</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>208224</v>
+        <v>237690</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K119" s="2" t="inlineStr">
         <is>
@@ -11952,10 +11952,10 @@
         <v>27294</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>257524</v>
+        <v>311968</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K120" s="2" t="inlineStr">
         <is>
@@ -12048,10 +12048,10 @@
         <v>27234</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>262086</v>
+        <v>305716</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K121" s="2" t="inlineStr">
         <is>
@@ -12240,10 +12240,10 @@
         <v>27042</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>204174</v>
+        <v>245644</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K123" s="2" t="inlineStr">
         <is>
@@ -12336,10 +12336,10 @@
         <v>26996</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>166437</v>
+        <v>188969</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K124" s="2" t="inlineStr">
         <is>
@@ -12432,10 +12432,10 @@
         <v>26814</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>340901</v>
+        <v>348711</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K125" s="2" t="inlineStr">
         <is>
@@ -12624,10 +12624,10 @@
         <v>26348</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>246549</v>
+        <v>299245</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
@@ -12720,10 +12720,10 @@
         <v>26286</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>144574</v>
+        <v>155570</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K128" s="2" t="inlineStr">
         <is>
@@ -12912,10 +12912,10 @@
         <v>26042</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>90666</v>
+        <v>119602</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
@@ -13008,10 +13008,10 @@
         <v>25641</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>147851</v>
+        <v>163545</v>
       </c>
       <c r="J131" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
@@ -13104,10 +13104,10 @@
         <v>25401</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>267550</v>
+        <v>273194</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K132" s="2" t="inlineStr">
         <is>
@@ -13200,10 +13200,10 @@
         <v>25381</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>163517</v>
+        <v>214279</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K133" s="2" t="inlineStr">
         <is>
@@ -13296,10 +13296,10 @@
         <v>25120</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>309566</v>
+        <v>334940</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K134" s="2" t="inlineStr">
         <is>
@@ -13392,10 +13392,10 @@
         <v>24466</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>244963</v>
+        <v>276769</v>
       </c>
       <c r="J135" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K135" s="2" t="inlineStr">
         <is>
@@ -13488,10 +13488,10 @@
         <v>24373</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>219732</v>
+        <v>256976</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K136" s="2" t="inlineStr">
         <is>
@@ -13584,10 +13584,10 @@
         <v>24370</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>322235</v>
+        <v>333655</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K137" s="2" t="inlineStr">
         <is>
@@ -13680,10 +13680,10 @@
         <v>23733</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>52682</v>
+        <v>63114</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K138" s="2" t="inlineStr">
         <is>
@@ -13776,10 +13776,10 @@
         <v>23700</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>82836</v>
+        <v>130236</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K139" s="2" t="inlineStr">
         <is>
@@ -13872,10 +13872,10 @@
         <v>23238</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>207723</v>
+        <v>254199</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K140" s="2" t="inlineStr">
         <is>
@@ -13968,10 +13968,10 @@
         <v>23199</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>68154</v>
+        <v>114552</v>
       </c>
       <c r="J141" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K141" s="2" t="inlineStr">
         <is>
@@ -14064,10 +14064,10 @@
         <v>23055</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>180299</v>
+        <v>192721</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
@@ -14160,10 +14160,10 @@
         <v>22693</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>27007</v>
+        <v>35635</v>
       </c>
       <c r="J143" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
@@ -14256,10 +14256,10 @@
         <v>22576</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>240160</v>
+        <v>285312</v>
       </c>
       <c r="J144" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
@@ -14352,10 +14352,10 @@
         <v>22178</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>130828</v>
+        <v>219540</v>
       </c>
       <c r="J145" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K145" s="2" t="inlineStr">
         <is>
@@ -14544,10 +14544,10 @@
         <v>21731</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>237110</v>
+        <v>259778</v>
       </c>
       <c r="J147" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K147" s="2" t="inlineStr">
         <is>
@@ -14640,10 +14640,10 @@
         <v>21717</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>154928</v>
+        <v>158090</v>
       </c>
       <c r="J148" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K148" s="2" t="inlineStr">
         <is>
@@ -14736,10 +14736,10 @@
         <v>21447</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>111532</v>
+        <v>154426</v>
       </c>
       <c r="J149" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K149" s="2" t="inlineStr">
         <is>
@@ -14832,10 +14832,10 @@
         <v>21410</v>
       </c>
       <c r="I150" s="2" t="n">
-        <v>243744</v>
+        <v>286564</v>
       </c>
       <c r="J150" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K150" s="2" t="inlineStr">
         <is>
@@ -14928,10 +14928,10 @@
         <v>21393</v>
       </c>
       <c r="I151" s="2" t="n">
-        <v>222350</v>
+        <v>225946</v>
       </c>
       <c r="J151" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K151" s="2" t="inlineStr">
         <is>
@@ -15024,10 +15024,10 @@
         <v>21379</v>
       </c>
       <c r="I152" s="2" t="n">
-        <v>154476</v>
+        <v>164122</v>
       </c>
       <c r="J152" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K152" s="2" t="inlineStr">
         <is>
@@ -15120,10 +15120,10 @@
         <v>21350</v>
       </c>
       <c r="I153" s="2" t="n">
-        <v>152682</v>
+        <v>164088</v>
       </c>
       <c r="J153" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K153" s="2" t="inlineStr">
         <is>
@@ -15216,10 +15216,10 @@
         <v>21292</v>
       </c>
       <c r="I154" s="2" t="n">
-        <v>245025</v>
+        <v>250883</v>
       </c>
       <c r="J154" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
@@ -15408,10 +15408,10 @@
         <v>21056</v>
       </c>
       <c r="I156" s="2" t="n">
-        <v>175674</v>
+        <v>203194</v>
       </c>
       <c r="J156" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
@@ -15504,10 +15504,10 @@
         <v>20991</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>158135</v>
+        <v>171801</v>
       </c>
       <c r="J157" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
@@ -15600,10 +15600,10 @@
         <v>20551</v>
       </c>
       <c r="I158" s="2" t="n">
-        <v>71956</v>
+        <v>113058</v>
       </c>
       <c r="J158" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K158" s="2" t="inlineStr">
         <is>
@@ -15696,10 +15696,10 @@
         <v>20138</v>
       </c>
       <c r="I159" s="2" t="n">
-        <v>138522</v>
+        <v>158208</v>
       </c>
       <c r="J159" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K159" s="2" t="inlineStr">
         <is>
@@ -15792,10 +15792,10 @@
         <v>20067</v>
       </c>
       <c r="I160" s="2" t="n">
-        <v>59347</v>
+        <v>99481</v>
       </c>
       <c r="J160" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K160" s="2" t="inlineStr">
         <is>
@@ -15888,10 +15888,10 @@
         <v>19798</v>
       </c>
       <c r="I161" s="2" t="n">
-        <v>196167</v>
+        <v>235763</v>
       </c>
       <c r="J161" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K161" s="2" t="inlineStr">
         <is>
@@ -16176,10 +16176,10 @@
         <v>19651</v>
       </c>
       <c r="I164" s="2" t="n">
-        <v>156816</v>
+        <v>172536</v>
       </c>
       <c r="J164" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K164" s="2" t="inlineStr">
         <is>
@@ -16464,10 +16464,10 @@
         <v>19421</v>
       </c>
       <c r="I167" s="2" t="n">
-        <v>19421</v>
+        <v>58263</v>
       </c>
       <c r="J167" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K167" s="2" t="inlineStr">
         <is>
@@ -16560,10 +16560,10 @@
         <v>19404</v>
       </c>
       <c r="I168" s="2" t="n">
-        <v>257882</v>
+        <v>293350</v>
       </c>
       <c r="J168" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K168" s="2" t="inlineStr">
         <is>
@@ -16656,10 +16656,10 @@
         <v>19350</v>
       </c>
       <c r="I169" s="2" t="n">
-        <v>133862</v>
+        <v>138362</v>
       </c>
       <c r="J169" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K169" s="2" t="inlineStr">
         <is>
@@ -16752,10 +16752,10 @@
         <v>19350</v>
       </c>
       <c r="I170" s="2" t="n">
-        <v>103050</v>
+        <v>105750</v>
       </c>
       <c r="J170" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K170" s="2" t="inlineStr">
         <is>
@@ -16848,10 +16848,10 @@
         <v>19326</v>
       </c>
       <c r="I171" s="2" t="n">
-        <v>49304</v>
+        <v>87956</v>
       </c>
       <c r="J171" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K171" s="2" t="inlineStr">
         <is>
@@ -17040,10 +17040,10 @@
         <v>19174</v>
       </c>
       <c r="I173" s="2" t="n">
-        <v>249262</v>
+        <v>287610</v>
       </c>
       <c r="J173" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K173" s="2" t="inlineStr">
         <is>
@@ -17136,10 +17136,10 @@
         <v>19173</v>
       </c>
       <c r="I174" s="2" t="n">
-        <v>184537</v>
+        <v>189329</v>
       </c>
       <c r="J174" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
@@ -17232,10 +17232,10 @@
         <v>19172</v>
       </c>
       <c r="I175" s="2" t="n">
-        <v>130849</v>
+        <v>162483</v>
       </c>
       <c r="J175" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K175" s="2" t="inlineStr">
         <is>
@@ -17328,10 +17328,10 @@
         <v>19075</v>
       </c>
       <c r="I176" s="2" t="n">
-        <v>202349</v>
+        <v>221243</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
@@ -17520,10 +17520,10 @@
         <v>18820</v>
       </c>
       <c r="I178" s="2" t="n">
-        <v>18820</v>
+        <v>56460</v>
       </c>
       <c r="J178" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
@@ -17616,10 +17616,10 @@
         <v>18691</v>
       </c>
       <c r="I179" s="2" t="n">
-        <v>81474</v>
+        <v>118856</v>
       </c>
       <c r="J179" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K179" s="2" t="inlineStr">
         <is>
@@ -17712,10 +17712,10 @@
         <v>18578</v>
       </c>
       <c r="I180" s="2" t="n">
-        <v>243968</v>
+        <v>265868</v>
       </c>
       <c r="J180" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K180" s="2" t="inlineStr">
         <is>
@@ -18000,10 +18000,10 @@
         <v>18435</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>174511</v>
+        <v>193917</v>
       </c>
       <c r="J183" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K183" s="2" t="inlineStr">
         <is>
@@ -18480,10 +18480,10 @@
         <v>17842</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>212503</v>
+        <v>248187</v>
       </c>
       <c r="J188" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K188" s="2" t="inlineStr">
         <is>
@@ -18576,10 +18576,10 @@
         <v>17796</v>
       </c>
       <c r="I189" s="2" t="n">
-        <v>191500</v>
+        <v>215180</v>
       </c>
       <c r="J189" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K189" s="2" t="inlineStr">
         <is>
@@ -18672,10 +18672,10 @@
         <v>17782</v>
       </c>
       <c r="I190" s="2" t="n">
-        <v>78038</v>
+        <v>113602</v>
       </c>
       <c r="J190" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
@@ -18768,10 +18768,10 @@
         <v>17780</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>88480</v>
+        <v>106400</v>
       </c>
       <c r="J191" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K191" s="2" t="inlineStr">
         <is>
@@ -18864,10 +18864,10 @@
         <v>17702</v>
       </c>
       <c r="I192" s="2" t="n">
-        <v>59468</v>
+        <v>94872</v>
       </c>
       <c r="J192" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
@@ -18960,10 +18960,10 @@
         <v>17677</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>143212</v>
+        <v>149140</v>
       </c>
       <c r="J193" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
@@ -19056,10 +19056,10 @@
         <v>17625</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>46793</v>
+        <v>82043</v>
       </c>
       <c r="J194" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
@@ -19152,10 +19152,10 @@
         <v>17525</v>
       </c>
       <c r="I195" s="2" t="n">
-        <v>88541</v>
+        <v>123591</v>
       </c>
       <c r="J195" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
@@ -19440,10 +19440,10 @@
         <v>17287</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>119065</v>
+        <v>153639</v>
       </c>
       <c r="J198" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K198" s="2" t="inlineStr">
         <is>
@@ -19536,10 +19536,10 @@
         <v>17116</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>131780</v>
+        <v>166012</v>
       </c>
       <c r="J199" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K199" s="2" t="inlineStr">
         <is>
@@ -19632,10 +19632,10 @@
         <v>17025</v>
       </c>
       <c r="I200" s="2" t="n">
-        <v>209150</v>
+        <v>234346</v>
       </c>
       <c r="J200" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K200" s="2" t="inlineStr">
         <is>
@@ -19728,10 +19728,10 @@
         <v>16937</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>50811</v>
+        <v>84685</v>
       </c>
       <c r="J201" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
@@ -19920,10 +19920,10 @@
         <v>16821</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>100258</v>
+        <v>115776</v>
       </c>
       <c r="J203" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
@@ -20112,10 +20112,10 @@
         <v>16587</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>154633</v>
+        <v>166371</v>
       </c>
       <c r="J205" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K205" s="2" t="inlineStr">
         <is>
@@ -20208,10 +20208,10 @@
         <v>16561</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>236442</v>
+        <v>269564</v>
       </c>
       <c r="J206" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K206" s="2" t="inlineStr">
         <is>
@@ -20304,10 +20304,10 @@
         <v>16561</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>113201</v>
+        <v>122963</v>
       </c>
       <c r="J207" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
@@ -20400,10 +20400,10 @@
         <v>16531</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>67988</v>
+        <v>97306</v>
       </c>
       <c r="J208" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K208" s="2" t="inlineStr">
         <is>
@@ -20496,10 +20496,10 @@
         <v>16494</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>122678</v>
+        <v>139608</v>
       </c>
       <c r="J209" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
@@ -20688,10 +20688,10 @@
         <v>16248</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>99246</v>
+        <v>131742</v>
       </c>
       <c r="J211" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K211" s="2" t="inlineStr">
         <is>
@@ -20784,10 +20784,10 @@
         <v>16166</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>186833</v>
+        <v>197279</v>
       </c>
       <c r="J212" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K212" s="2" t="inlineStr">
         <is>
@@ -20880,10 +20880,10 @@
         <v>16126</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>136647</v>
+        <v>168899</v>
       </c>
       <c r="J213" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K213" s="2" t="inlineStr">
         <is>
@@ -20976,10 +20976,10 @@
         <v>16043</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>125095</v>
+        <v>134623</v>
       </c>
       <c r="J214" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K214" s="2" t="inlineStr">
         <is>
@@ -21072,10 +21072,10 @@
         <v>16013</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>94809</v>
+        <v>102035</v>
       </c>
       <c r="J215" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
@@ -21168,10 +21168,10 @@
         <v>15938</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>126644</v>
+        <v>158520</v>
       </c>
       <c r="J216" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
@@ -21264,10 +21264,10 @@
         <v>15807</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>220827</v>
+        <v>236635</v>
       </c>
       <c r="J217" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K217" s="2" t="inlineStr">
         <is>
@@ -21360,10 +21360,10 @@
         <v>15719</v>
       </c>
       <c r="I218" s="2" t="n">
-        <v>15719</v>
+        <v>47157</v>
       </c>
       <c r="J218" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K218" s="2" t="inlineStr">
         <is>
@@ -21648,10 +21648,10 @@
         <v>15275</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>69935</v>
+        <v>100485</v>
       </c>
       <c r="J221" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K221" s="2" t="inlineStr">
         <is>
@@ -21744,10 +21744,10 @@
         <v>15075</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>95355</v>
+        <v>98213</v>
       </c>
       <c r="J222" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K222" s="2" t="inlineStr">
         <is>
@@ -21840,10 +21840,10 @@
         <v>14953</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>127041</v>
+        <v>132117</v>
       </c>
       <c r="J223" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K223" s="2" t="inlineStr">
         <is>
@@ -22032,10 +22032,10 @@
         <v>14869</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>119522</v>
+        <v>149260</v>
       </c>
       <c r="J225" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
@@ -22128,10 +22128,10 @@
         <v>14646</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>96593</v>
+        <v>125885</v>
       </c>
       <c r="J226" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K226" s="2" t="inlineStr">
         <is>
@@ -22320,10 +22320,10 @@
         <v>14628</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>14628</v>
+        <v>43884</v>
       </c>
       <c r="J228" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K228" s="2" t="inlineStr">
         <is>
@@ -22512,10 +22512,10 @@
         <v>14436</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>137219</v>
+        <v>160593</v>
       </c>
       <c r="J230" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K230" s="2" t="inlineStr">
         <is>
@@ -22800,10 +22800,10 @@
         <v>14380</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>33538</v>
+        <v>62298</v>
       </c>
       <c r="J233" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K233" s="2" t="inlineStr">
         <is>
@@ -22896,10 +22896,10 @@
         <v>14313</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>175900</v>
+        <v>191654</v>
       </c>
       <c r="J234" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K234" s="2" t="inlineStr">
         <is>
@@ -22992,10 +22992,10 @@
         <v>14313</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>59573</v>
+        <v>88199</v>
       </c>
       <c r="J235" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K235" s="2" t="inlineStr">
         <is>
@@ -23088,10 +23088,10 @@
         <v>14257</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>65579</v>
+        <v>94093</v>
       </c>
       <c r="J236" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
@@ -23184,10 +23184,10 @@
         <v>14158</v>
       </c>
       <c r="I237" s="2" t="n">
-        <v>30558</v>
+        <v>58874</v>
       </c>
       <c r="J237" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K237" s="2" t="inlineStr">
         <is>
@@ -23376,10 +23376,10 @@
         <v>14149</v>
       </c>
       <c r="I239" s="2" t="n">
-        <v>197744</v>
+        <v>209318</v>
       </c>
       <c r="J239" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K239" s="2" t="inlineStr">
         <is>
@@ -23472,10 +23472,10 @@
         <v>14114</v>
       </c>
       <c r="I240" s="2" t="n">
-        <v>37637</v>
+        <v>56455</v>
       </c>
       <c r="J240" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K240" s="2" t="inlineStr">
         <is>
@@ -23760,10 +23760,10 @@
         <v>14097</v>
       </c>
       <c r="I243" s="2" t="n">
-        <v>746140</v>
+        <v>760280</v>
       </c>
       <c r="J243" s="2" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K243" s="2" t="inlineStr">
         <is>
@@ -23856,10 +23856,10 @@
         <v>14042</v>
       </c>
       <c r="I244" s="2" t="n">
-        <v>106503</v>
+        <v>123491</v>
       </c>
       <c r="J244" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K244" s="2" t="inlineStr">
         <is>
@@ -24048,10 +24048,10 @@
         <v>13912</v>
       </c>
       <c r="I246" s="2" t="n">
-        <v>177879</v>
+        <v>181925</v>
       </c>
       <c r="J246" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K246" s="2" t="inlineStr">
         <is>
@@ -24336,10 +24336,10 @@
         <v>13768</v>
       </c>
       <c r="I249" s="2" t="n">
-        <v>41930</v>
+        <v>54168</v>
       </c>
       <c r="J249" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K249" s="2" t="inlineStr">
         <is>
@@ -24432,10 +24432,10 @@
         <v>13641</v>
       </c>
       <c r="I250" s="2" t="n">
-        <v>88431</v>
+        <v>111949</v>
       </c>
       <c r="J250" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K250" s="2" t="inlineStr">
         <is>
@@ -24528,10 +24528,10 @@
         <v>13563</v>
       </c>
       <c r="I251" s="2" t="n">
-        <v>111684</v>
+        <v>117542</v>
       </c>
       <c r="J251" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K251" s="2" t="inlineStr">
         <is>
@@ -24624,10 +24624,10 @@
         <v>13541</v>
       </c>
       <c r="I252" s="2" t="n">
-        <v>166714</v>
+        <v>175624</v>
       </c>
       <c r="J252" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K252" s="2" t="inlineStr">
         <is>
@@ -24720,10 +24720,10 @@
         <v>13504</v>
       </c>
       <c r="I253" s="2" t="n">
-        <v>40512</v>
+        <v>67520</v>
       </c>
       <c r="J253" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K253" s="2" t="inlineStr">
         <is>
@@ -25200,10 +25200,10 @@
         <v>13172</v>
       </c>
       <c r="I258" s="2" t="n">
-        <v>173585</v>
+        <v>176407</v>
       </c>
       <c r="J258" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K258" s="2" t="inlineStr">
         <is>
@@ -25296,10 +25296,10 @@
         <v>12786</v>
       </c>
       <c r="I259" s="2" t="n">
-        <v>134471</v>
+        <v>141835</v>
       </c>
       <c r="J259" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K259" s="2" t="inlineStr">
         <is>
@@ -25392,10 +25392,10 @@
         <v>12745</v>
       </c>
       <c r="I260" s="2" t="n">
-        <v>68244</v>
+        <v>93734</v>
       </c>
       <c r="J260" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K260" s="2" t="inlineStr">
         <is>
@@ -25584,10 +25584,10 @@
         <v>12689</v>
       </c>
       <c r="I262" s="2" t="n">
-        <v>115178</v>
+        <v>130794</v>
       </c>
       <c r="J262" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K262" s="2" t="inlineStr">
         <is>
@@ -25776,10 +25776,10 @@
         <v>12382</v>
       </c>
       <c r="I264" s="2" t="n">
-        <v>34605</v>
+        <v>44381</v>
       </c>
       <c r="J264" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K264" s="2" t="inlineStr">
         <is>
@@ -25872,10 +25872,10 @@
         <v>12340</v>
       </c>
       <c r="I265" s="2" t="n">
-        <v>94563</v>
+        <v>110929</v>
       </c>
       <c r="J265" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K265" s="2" t="inlineStr">
         <is>
@@ -25968,10 +25968,10 @@
         <v>12303</v>
       </c>
       <c r="I266" s="2" t="n">
-        <v>174547</v>
+        <v>185123</v>
       </c>
       <c r="J266" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K266" s="2" t="inlineStr">
         <is>
@@ -26064,10 +26064,10 @@
         <v>12156</v>
       </c>
       <c r="I267" s="2" t="n">
-        <v>38996</v>
+        <v>43876</v>
       </c>
       <c r="J267" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K267" s="2" t="inlineStr">
         <is>
@@ -26160,10 +26160,10 @@
         <v>12149</v>
       </c>
       <c r="I268" s="2" t="n">
-        <v>75464</v>
+        <v>99762</v>
       </c>
       <c r="J268" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K268" s="2" t="inlineStr">
         <is>
@@ -26544,10 +26544,10 @@
         <v>11619</v>
       </c>
       <c r="I272" s="2" t="n">
-        <v>112708</v>
+        <v>135946</v>
       </c>
       <c r="J272" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K272" s="2" t="inlineStr">
         <is>
@@ -26928,10 +26928,10 @@
         <v>11284</v>
       </c>
       <c r="I276" s="2" t="n">
-        <v>113833</v>
+        <v>117589</v>
       </c>
       <c r="J276" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K276" s="2" t="inlineStr">
         <is>
@@ -27024,10 +27024,10 @@
         <v>11226</v>
       </c>
       <c r="I277" s="2" t="n">
-        <v>82262</v>
+        <v>87142</v>
       </c>
       <c r="J277" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K277" s="2" t="inlineStr">
         <is>
@@ -27120,10 +27120,10 @@
         <v>10989</v>
       </c>
       <c r="I278" s="2" t="n">
-        <v>101025</v>
+        <v>103901</v>
       </c>
       <c r="J278" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K278" s="2" t="inlineStr">
         <is>
@@ -27216,10 +27216,10 @@
         <v>10726</v>
       </c>
       <c r="I279" s="2" t="n">
-        <v>114878</v>
+        <v>136330</v>
       </c>
       <c r="J279" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K279" s="2" t="inlineStr">
         <is>
@@ -27312,10 +27312,10 @@
         <v>10675</v>
       </c>
       <c r="I280" s="2" t="n">
-        <v>29167</v>
+        <v>44801</v>
       </c>
       <c r="J280" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K280" s="2" t="inlineStr">
         <is>
@@ -27408,10 +27408,10 @@
         <v>10673</v>
       </c>
       <c r="I281" s="2" t="n">
-        <v>128754</v>
+        <v>150100</v>
       </c>
       <c r="J281" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K281" s="2" t="inlineStr">
         <is>
@@ -27504,10 +27504,10 @@
         <v>10641</v>
       </c>
       <c r="I282" s="2" t="n">
-        <v>21073</v>
+        <v>42355</v>
       </c>
       <c r="J282" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K282" s="2" t="inlineStr">
         <is>
@@ -27600,10 +27600,10 @@
         <v>10325</v>
       </c>
       <c r="I283" s="2" t="n">
-        <v>35450</v>
+        <v>40694</v>
       </c>
       <c r="J283" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K283" s="2" t="inlineStr">
         <is>
@@ -27792,10 +27792,10 @@
         <v>10306</v>
       </c>
       <c r="I285" s="2" t="n">
-        <v>55685</v>
+        <v>71961</v>
       </c>
       <c r="J285" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K285" s="2" t="inlineStr">
         <is>
@@ -27888,10 +27888,10 @@
         <v>10268</v>
       </c>
       <c r="I286" s="2" t="n">
-        <v>87298</v>
+        <v>102116</v>
       </c>
       <c r="J286" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K286" s="2" t="inlineStr">
         <is>
@@ -27984,10 +27984,10 @@
         <v>10190</v>
       </c>
       <c r="I287" s="2" t="n">
-        <v>84917</v>
+        <v>102387</v>
       </c>
       <c r="J287" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K287" s="2" t="inlineStr">
         <is>
@@ -28080,10 +28080,10 @@
         <v>10127</v>
       </c>
       <c r="I288" s="2" t="n">
-        <v>32870</v>
+        <v>36724</v>
       </c>
       <c r="J288" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K288" s="2" t="inlineStr">
         <is>
@@ -28368,10 +28368,10 @@
         <v>10057</v>
       </c>
       <c r="I291" s="2" t="n">
-        <v>119275</v>
+        <v>128257</v>
       </c>
       <c r="J291" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K291" s="2" t="inlineStr">
         <is>
@@ -28752,10 +28752,10 @@
         <v>9881</v>
       </c>
       <c r="I295" s="2" t="n">
-        <v>174613</v>
+        <v>193785</v>
       </c>
       <c r="J295" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K295" s="2" t="inlineStr">
         <is>
@@ -28944,10 +28944,10 @@
         <v>9863</v>
       </c>
       <c r="I297" s="2" t="n">
-        <v>100742</v>
+        <v>112014</v>
       </c>
       <c r="J297" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K297" s="2" t="inlineStr">
         <is>
@@ -29040,10 +29040,10 @@
         <v>9823</v>
       </c>
       <c r="I298" s="2" t="n">
-        <v>68807</v>
+        <v>75093</v>
       </c>
       <c r="J298" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K298" s="2" t="inlineStr">
         <is>
@@ -29136,10 +29136,10 @@
         <v>9814</v>
       </c>
       <c r="I299" s="2" t="n">
-        <v>76157</v>
+        <v>93633</v>
       </c>
       <c r="J299" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K299" s="2" t="inlineStr">
         <is>
@@ -29232,10 +29232,10 @@
         <v>9813</v>
       </c>
       <c r="I300" s="2" t="n">
-        <v>29439</v>
+        <v>49065</v>
       </c>
       <c r="J300" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K300" s="2" t="inlineStr">
         <is>
@@ -29328,10 +29328,10 @@
         <v>9795</v>
       </c>
       <c r="I301" s="2" t="n">
-        <v>58284</v>
+        <v>73956</v>
       </c>
       <c r="J301" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K301" s="2" t="inlineStr">
         <is>
@@ -29424,10 +29424,10 @@
         <v>9763</v>
       </c>
       <c r="I302" s="2" t="n">
-        <v>9763</v>
+        <v>29289</v>
       </c>
       <c r="J302" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K302" s="2" t="inlineStr">
         <is>
@@ -29904,10 +29904,10 @@
         <v>9631</v>
       </c>
       <c r="I307" s="2" t="n">
-        <v>40462</v>
+        <v>53942</v>
       </c>
       <c r="J307" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K307" s="2" t="inlineStr">
         <is>
@@ -30000,10 +30000,10 @@
         <v>9608</v>
       </c>
       <c r="I308" s="2" t="n">
-        <v>23626</v>
+        <v>26326</v>
       </c>
       <c r="J308" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K308" s="2" t="inlineStr">
         <is>
@@ -30096,10 +30096,10 @@
         <v>9587</v>
       </c>
       <c r="I309" s="2" t="n">
-        <v>99968</v>
+        <v>104858</v>
       </c>
       <c r="J309" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K309" s="2" t="inlineStr">
         <is>
@@ -30288,10 +30288,10 @@
         <v>9586</v>
       </c>
       <c r="I311" s="2" t="n">
-        <v>112540</v>
+        <v>122126</v>
       </c>
       <c r="J311" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K311" s="2" t="inlineStr">
         <is>
@@ -30576,10 +30576,10 @@
         <v>9470</v>
       </c>
       <c r="I314" s="2" t="n">
-        <v>135735</v>
+        <v>148323</v>
       </c>
       <c r="J314" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K314" s="2" t="inlineStr">
         <is>
@@ -30672,10 +30672,10 @@
         <v>9348</v>
       </c>
       <c r="I315" s="2" t="n">
-        <v>98329</v>
+        <v>108027</v>
       </c>
       <c r="J315" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K315" s="2" t="inlineStr">
         <is>
@@ -30768,10 +30768,10 @@
         <v>9306</v>
       </c>
       <c r="I316" s="2" t="n">
-        <v>88881</v>
+        <v>107493</v>
       </c>
       <c r="J316" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K316" s="2" t="inlineStr">
         <is>
@@ -30864,10 +30864,10 @@
         <v>9274</v>
       </c>
       <c r="I317" s="2" t="n">
-        <v>88762</v>
+        <v>107310</v>
       </c>
       <c r="J317" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K317" s="2" t="inlineStr">
         <is>
@@ -30960,10 +30960,10 @@
         <v>9236</v>
       </c>
       <c r="I318" s="2" t="n">
-        <v>32069</v>
+        <v>35153</v>
       </c>
       <c r="J318" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K318" s="2" t="inlineStr">
         <is>
@@ -31248,10 +31248,10 @@
         <v>9072</v>
       </c>
       <c r="I321" s="2" t="n">
-        <v>23270</v>
+        <v>41414</v>
       </c>
       <c r="J321" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
@@ -31344,10 +31344,10 @@
         <v>9047</v>
       </c>
       <c r="I322" s="2" t="n">
-        <v>69446</v>
+        <v>81916</v>
       </c>
       <c r="J322" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
@@ -31440,10 +31440,10 @@
         <v>9028</v>
       </c>
       <c r="I323" s="2" t="n">
-        <v>32531</v>
+        <v>37865</v>
       </c>
       <c r="J323" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K323" s="2" t="inlineStr">
         <is>
@@ -31632,10 +31632,10 @@
         <v>8932</v>
       </c>
       <c r="I325" s="2" t="n">
-        <v>8932</v>
+        <v>26796</v>
       </c>
       <c r="J325" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K325" s="2" t="inlineStr">
         <is>
@@ -31728,10 +31728,10 @@
         <v>8893</v>
       </c>
       <c r="I326" s="2" t="n">
-        <v>80521</v>
+        <v>85461</v>
       </c>
       <c r="J326" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K326" s="2" t="inlineStr">
         <is>
@@ -31920,10 +31920,10 @@
         <v>8847</v>
       </c>
       <c r="I328" s="2" t="n">
-        <v>123466</v>
+        <v>139840</v>
       </c>
       <c r="J328" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K328" s="2" t="inlineStr">
         <is>
@@ -32208,10 +32208,10 @@
         <v>8788</v>
       </c>
       <c r="I331" s="2" t="n">
-        <v>22169</v>
+        <v>31355</v>
       </c>
       <c r="J331" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
@@ -32400,10 +32400,10 @@
         <v>8726</v>
       </c>
       <c r="I333" s="2" t="n">
-        <v>143187</v>
+        <v>148061</v>
       </c>
       <c r="J333" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K333" s="2" t="inlineStr">
         <is>
@@ -32688,10 +32688,10 @@
         <v>8644</v>
       </c>
       <c r="I336" s="2" t="n">
-        <v>46487</v>
+        <v>53155</v>
       </c>
       <c r="J336" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K336" s="2" t="inlineStr">
         <is>
@@ -32784,10 +32784,10 @@
         <v>8643</v>
       </c>
       <c r="I337" s="2" t="n">
-        <v>32871</v>
+        <v>39623</v>
       </c>
       <c r="J337" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K337" s="2" t="inlineStr">
         <is>
@@ -32880,10 +32880,10 @@
         <v>8585</v>
       </c>
       <c r="I338" s="2" t="n">
-        <v>74594</v>
+        <v>80352</v>
       </c>
       <c r="J338" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
@@ -32976,10 +32976,10 @@
         <v>8561</v>
       </c>
       <c r="I339" s="2" t="n">
-        <v>88713</v>
+        <v>94919</v>
       </c>
       <c r="J339" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K339" s="2" t="inlineStr">
         <is>
@@ -33072,10 +33072,10 @@
         <v>8540</v>
       </c>
       <c r="I340" s="2" t="n">
-        <v>65008</v>
+        <v>98754</v>
       </c>
       <c r="J340" s="2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K340" s="2" t="inlineStr">
         <is>
@@ -33168,10 +33168,10 @@
         <v>8467</v>
       </c>
       <c r="I341" s="2" t="n">
-        <v>56445</v>
+        <v>63969</v>
       </c>
       <c r="J341" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K341" s="2" t="inlineStr">
         <is>
@@ -33552,10 +33552,10 @@
         <v>8151</v>
       </c>
       <c r="I345" s="2" t="n">
-        <v>20182</v>
+        <v>27942</v>
       </c>
       <c r="J345" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K345" s="2" t="inlineStr">
         <is>
@@ -33840,10 +33840,10 @@
         <v>8136</v>
       </c>
       <c r="I348" s="2" t="n">
-        <v>28386</v>
+        <v>44658</v>
       </c>
       <c r="J348" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K348" s="2" t="inlineStr">
         <is>
@@ -34320,10 +34320,10 @@
         <v>7997</v>
       </c>
       <c r="I353" s="2" t="n">
-        <v>40163</v>
+        <v>56157</v>
       </c>
       <c r="J353" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K353" s="2" t="inlineStr">
         <is>
@@ -34512,10 +34512,10 @@
         <v>7809</v>
       </c>
       <c r="I355" s="2" t="n">
-        <v>50691</v>
+        <v>66167</v>
       </c>
       <c r="J355" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K355" s="2" t="inlineStr">
         <is>
@@ -34608,10 +34608,10 @@
         <v>7763</v>
       </c>
       <c r="I356" s="2" t="n">
-        <v>7763</v>
+        <v>23289</v>
       </c>
       <c r="J356" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
@@ -34800,10 +34800,10 @@
         <v>7713</v>
       </c>
       <c r="I358" s="2" t="n">
-        <v>95934</v>
+        <v>99790</v>
       </c>
       <c r="J358" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K358" s="2" t="inlineStr">
         <is>
@@ -34992,10 +34992,10 @@
         <v>7564</v>
       </c>
       <c r="I360" s="2" t="n">
-        <v>13458</v>
+        <v>28586</v>
       </c>
       <c r="J360" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
@@ -35088,10 +35088,10 @@
         <v>7560</v>
       </c>
       <c r="I361" s="2" t="n">
-        <v>20160</v>
+        <v>30240</v>
       </c>
       <c r="J361" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K361" s="2" t="inlineStr">
         <is>
@@ -35280,10 +35280,10 @@
         <v>7524</v>
       </c>
       <c r="I363" s="2" t="n">
-        <v>20691</v>
+        <v>35739</v>
       </c>
       <c r="J363" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K363" s="2" t="inlineStr">
         <is>
@@ -35664,10 +35664,10 @@
         <v>7428</v>
       </c>
       <c r="I367" s="2" t="n">
-        <v>43431</v>
+        <v>47241</v>
       </c>
       <c r="J367" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K367" s="2" t="inlineStr">
         <is>
@@ -35856,10 +35856,10 @@
         <v>7223</v>
       </c>
       <c r="I369" s="2" t="n">
-        <v>66054</v>
+        <v>73278</v>
       </c>
       <c r="J369" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K369" s="2" t="inlineStr">
         <is>
@@ -36336,10 +36336,10 @@
         <v>7074</v>
       </c>
       <c r="I374" s="2" t="n">
-        <v>82095</v>
+        <v>92517</v>
       </c>
       <c r="J374" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K374" s="2" t="inlineStr">
         <is>
@@ -36432,10 +36432,10 @@
         <v>7073</v>
       </c>
       <c r="I375" s="2" t="n">
-        <v>7073</v>
+        <v>21219</v>
       </c>
       <c r="J375" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K375" s="2" t="inlineStr">
         <is>
@@ -36720,10 +36720,10 @@
         <v>6875</v>
       </c>
       <c r="I378" s="2" t="n">
-        <v>44075</v>
+        <v>57589</v>
       </c>
       <c r="J378" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K378" s="2" t="inlineStr">
         <is>
@@ -36816,10 +36816,10 @@
         <v>6835</v>
       </c>
       <c r="I379" s="2" t="n">
-        <v>50774</v>
+        <v>56632</v>
       </c>
       <c r="J379" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K379" s="2" t="inlineStr">
         <is>
@@ -36912,10 +36912,10 @@
         <v>6833</v>
       </c>
       <c r="I380" s="2" t="n">
-        <v>16594</v>
+        <v>22450</v>
       </c>
       <c r="J380" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K380" s="2" t="inlineStr">
         <is>
@@ -37008,10 +37008,10 @@
         <v>6752</v>
       </c>
       <c r="I381" s="2" t="n">
-        <v>53536</v>
+        <v>58360</v>
       </c>
       <c r="J381" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K381" s="2" t="inlineStr">
         <is>
@@ -37104,10 +37104,10 @@
         <v>6751</v>
       </c>
       <c r="I382" s="2" t="n">
-        <v>6751</v>
+        <v>20253</v>
       </c>
       <c r="J382" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K382" s="2" t="inlineStr">
         <is>
@@ -37200,10 +37200,10 @@
         <v>6750</v>
       </c>
       <c r="I383" s="2" t="n">
-        <v>50625</v>
+        <v>57375</v>
       </c>
       <c r="J383" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K383" s="2" t="inlineStr">
         <is>
@@ -37296,10 +37296,10 @@
         <v>6666</v>
       </c>
       <c r="I384" s="2" t="n">
-        <v>29522</v>
+        <v>42854</v>
       </c>
       <c r="J384" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K384" s="2" t="inlineStr">
         <is>
@@ -37584,10 +37584,10 @@
         <v>6585</v>
       </c>
       <c r="I387" s="2" t="n">
-        <v>75721</v>
+        <v>84191</v>
       </c>
       <c r="J387" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K387" s="2" t="inlineStr">
         <is>
@@ -37680,10 +37680,10 @@
         <v>6585</v>
       </c>
       <c r="I388" s="2" t="n">
-        <v>39509</v>
+        <v>47035</v>
       </c>
       <c r="J388" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K388" s="2" t="inlineStr">
         <is>
@@ -37776,10 +37776,10 @@
         <v>6578</v>
       </c>
       <c r="I389" s="2" t="n">
-        <v>48370</v>
+        <v>52242</v>
       </c>
       <c r="J389" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K389" s="2" t="inlineStr">
         <is>
@@ -37872,10 +37872,10 @@
         <v>6575</v>
       </c>
       <c r="I390" s="2" t="n">
-        <v>30562</v>
+        <v>43712</v>
       </c>
       <c r="J390" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K390" s="2" t="inlineStr">
         <is>
@@ -38064,10 +38064,10 @@
         <v>6522</v>
       </c>
       <c r="I392" s="2" t="n">
-        <v>81472</v>
+        <v>91592</v>
       </c>
       <c r="J392" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K392" s="2" t="inlineStr">
         <is>
@@ -38352,10 +38352,10 @@
         <v>6469</v>
       </c>
       <c r="I395" s="2" t="n">
-        <v>72637</v>
+        <v>83411</v>
       </c>
       <c r="J395" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K395" s="2" t="inlineStr">
         <is>
@@ -38544,10 +38544,10 @@
         <v>6402</v>
       </c>
       <c r="I397" s="2" t="n">
-        <v>13864</v>
+        <v>15984</v>
       </c>
       <c r="J397" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K397" s="2" t="inlineStr">
         <is>
@@ -38928,10 +38928,10 @@
         <v>6286</v>
       </c>
       <c r="I401" s="2" t="n">
-        <v>33877</v>
+        <v>43507</v>
       </c>
       <c r="J401" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K401" s="2" t="inlineStr">
         <is>
@@ -39024,10 +39024,10 @@
         <v>6286</v>
       </c>
       <c r="I402" s="2" t="n">
-        <v>55788</v>
+        <v>66788</v>
       </c>
       <c r="J402" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K402" s="2" t="inlineStr">
         <is>
@@ -39120,10 +39120,10 @@
         <v>6285</v>
       </c>
       <c r="I403" s="2" t="n">
-        <v>37334</v>
+        <v>43810</v>
       </c>
       <c r="J403" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K403" s="2" t="inlineStr">
         <is>
@@ -39216,10 +39216,10 @@
         <v>6269</v>
       </c>
       <c r="I404" s="2" t="n">
-        <v>68477</v>
+        <v>80051</v>
       </c>
       <c r="J404" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K404" s="2" t="inlineStr">
         <is>
@@ -39312,10 +39312,10 @@
         <v>6232</v>
       </c>
       <c r="I405" s="2" t="n">
-        <v>50852</v>
+        <v>63316</v>
       </c>
       <c r="J405" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K405" s="2" t="inlineStr">
         <is>
@@ -39696,10 +39696,10 @@
         <v>6047</v>
       </c>
       <c r="I409" s="2" t="n">
-        <v>35269</v>
+        <v>39141</v>
       </c>
       <c r="J409" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K409" s="2" t="inlineStr">
         <is>
@@ -39792,10 +39792,10 @@
         <v>5956</v>
       </c>
       <c r="I410" s="2" t="n">
-        <v>28021</v>
+        <v>36809</v>
       </c>
       <c r="J410" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K410" s="2" t="inlineStr">
         <is>
@@ -39984,10 +39984,10 @@
         <v>5912</v>
       </c>
       <c r="I412" s="2" t="n">
-        <v>19434</v>
+        <v>31258</v>
       </c>
       <c r="J412" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K412" s="2" t="inlineStr">
         <is>
@@ -40176,10 +40176,10 @@
         <v>5857</v>
       </c>
       <c r="I414" s="2" t="n">
-        <v>54487</v>
+        <v>66201</v>
       </c>
       <c r="J414" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K414" s="2" t="inlineStr">
         <is>
@@ -40368,10 +40368,10 @@
         <v>5846</v>
       </c>
       <c r="I416" s="2" t="n">
-        <v>54776</v>
+        <v>62084</v>
       </c>
       <c r="J416" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K416" s="2" t="inlineStr">
         <is>
@@ -40560,10 +40560,10 @@
         <v>5834</v>
       </c>
       <c r="I418" s="2" t="n">
-        <v>59657</v>
+        <v>62291</v>
       </c>
       <c r="J418" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K418" s="2" t="inlineStr">
         <is>
@@ -40752,10 +40752,10 @@
         <v>5782</v>
       </c>
       <c r="I420" s="2" t="n">
-        <v>22764</v>
+        <v>34328</v>
       </c>
       <c r="J420" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K420" s="2" t="inlineStr">
         <is>
@@ -40944,10 +40944,10 @@
         <v>5717</v>
       </c>
       <c r="I422" s="2" t="n">
-        <v>41924</v>
+        <v>51452</v>
       </c>
       <c r="J422" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K422" s="2" t="inlineStr">
         <is>
@@ -41040,10 +41040,10 @@
         <v>5674</v>
       </c>
       <c r="I423" s="2" t="n">
-        <v>63724</v>
+        <v>72260</v>
       </c>
       <c r="J423" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K423" s="2" t="inlineStr">
         <is>
@@ -41232,10 +41232,10 @@
         <v>5643</v>
       </c>
       <c r="I425" s="2" t="n">
-        <v>66840</v>
+        <v>78126</v>
       </c>
       <c r="J425" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K425" s="2" t="inlineStr">
         <is>
@@ -41328,10 +41328,10 @@
         <v>5643</v>
       </c>
       <c r="I426" s="2" t="n">
-        <v>26808</v>
+        <v>38094</v>
       </c>
       <c r="J426" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K426" s="2" t="inlineStr">
         <is>
@@ -41808,10 +41808,10 @@
         <v>5420</v>
       </c>
       <c r="I431" s="2" t="n">
-        <v>70512</v>
+        <v>72690</v>
       </c>
       <c r="J431" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K431" s="2" t="inlineStr">
         <is>
@@ -42000,10 +42000,10 @@
         <v>5400</v>
       </c>
       <c r="I433" s="2" t="n">
-        <v>34681</v>
+        <v>38539</v>
       </c>
       <c r="J433" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K433" s="2" t="inlineStr">
         <is>
@@ -42192,10 +42192,10 @@
         <v>5397</v>
       </c>
       <c r="I435" s="2" t="n">
-        <v>58017</v>
+        <v>60715</v>
       </c>
       <c r="J435" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K435" s="2" t="inlineStr">
         <is>
@@ -42288,10 +42288,10 @@
         <v>5396</v>
       </c>
       <c r="I436" s="2" t="n">
-        <v>40470</v>
+        <v>45866</v>
       </c>
       <c r="J436" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K436" s="2" t="inlineStr">
         <is>
@@ -42480,10 +42480,10 @@
         <v>5389</v>
       </c>
       <c r="I438" s="2" t="n">
-        <v>52295</v>
+        <v>59361</v>
       </c>
       <c r="J438" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K438" s="2" t="inlineStr">
         <is>
@@ -42672,10 +42672,10 @@
         <v>5271</v>
       </c>
       <c r="I440" s="2" t="n">
-        <v>39744</v>
+        <v>50286</v>
       </c>
       <c r="J440" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K440" s="2" t="inlineStr">
         <is>
@@ -42768,10 +42768,10 @@
         <v>5270</v>
       </c>
       <c r="I441" s="2" t="n">
-        <v>76547</v>
+        <v>82213</v>
       </c>
       <c r="J441" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K441" s="2" t="inlineStr">
         <is>
@@ -42864,10 +42864,10 @@
         <v>5268</v>
       </c>
       <c r="I442" s="2" t="n">
-        <v>27846</v>
+        <v>38382</v>
       </c>
       <c r="J442" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K442" s="2" t="inlineStr">
         <is>
@@ -42960,10 +42960,10 @@
         <v>5259</v>
       </c>
       <c r="I443" s="2" t="n">
-        <v>5259</v>
+        <v>15777</v>
       </c>
       <c r="J443" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K443" s="2" t="inlineStr">
         <is>
@@ -43344,10 +43344,10 @@
         <v>5176</v>
       </c>
       <c r="I447" s="2" t="n">
-        <v>60699</v>
+        <v>71051</v>
       </c>
       <c r="J447" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K447" s="2" t="inlineStr">
         <is>
@@ -43632,10 +43632,10 @@
         <v>5125</v>
       </c>
       <c r="I450" s="2" t="n">
-        <v>5125</v>
+        <v>15375</v>
       </c>
       <c r="J450" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K450" s="2" t="inlineStr">
         <is>
@@ -43728,10 +43728,10 @@
         <v>5101</v>
       </c>
       <c r="I451" s="2" t="n">
-        <v>5101</v>
+        <v>15303</v>
       </c>
       <c r="J451" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K451" s="2" t="inlineStr">
         <is>
@@ -43920,10 +43920,10 @@
         <v>5027</v>
       </c>
       <c r="I453" s="2" t="n">
-        <v>51016</v>
+        <v>56058</v>
       </c>
       <c r="J453" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K453" s="2" t="inlineStr">
         <is>
@@ -44016,10 +44016,10 @@
         <v>5004</v>
       </c>
       <c r="I454" s="2" t="n">
-        <v>21019</v>
+        <v>25023</v>
       </c>
       <c r="J454" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K454" s="2" t="inlineStr">
         <is>
@@ -44208,10 +44208,10 @@
         <v>4911</v>
       </c>
       <c r="I456" s="2" t="n">
-        <v>36335</v>
+        <v>46157</v>
       </c>
       <c r="J456" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K456" s="2" t="inlineStr">
         <is>
@@ -44496,10 +44496,10 @@
         <v>4881</v>
       </c>
       <c r="I459" s="2" t="n">
-        <v>4881</v>
+        <v>14643</v>
       </c>
       <c r="J459" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K459" s="2" t="inlineStr">
         <is>
@@ -44688,10 +44688,10 @@
         <v>4869</v>
       </c>
       <c r="I461" s="2" t="n">
-        <v>42268</v>
+        <v>49052</v>
       </c>
       <c r="J461" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K461" s="2" t="inlineStr">
         <is>
@@ -44784,10 +44784,10 @@
         <v>4853</v>
       </c>
       <c r="I462" s="2" t="n">
-        <v>62603</v>
+        <v>72309</v>
       </c>
       <c r="J462" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K462" s="2" t="inlineStr">
         <is>
@@ -44880,10 +44880,10 @@
         <v>4853</v>
       </c>
       <c r="I463" s="2" t="n">
-        <v>11647</v>
+        <v>15529</v>
       </c>
       <c r="J463" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K463" s="2" t="inlineStr">
         <is>
@@ -45072,10 +45072,10 @@
         <v>4851</v>
       </c>
       <c r="I465" s="2" t="n">
-        <v>23766</v>
+        <v>33468</v>
       </c>
       <c r="J465" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K465" s="2" t="inlineStr">
         <is>
@@ -45168,10 +45168,10 @@
         <v>4845</v>
       </c>
       <c r="I466" s="2" t="n">
-        <v>54264</v>
+        <v>60078</v>
       </c>
       <c r="J466" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K466" s="2" t="inlineStr">
         <is>
@@ -45360,10 +45360,10 @@
         <v>4822</v>
       </c>
       <c r="I468" s="2" t="n">
-        <v>40986</v>
+        <v>50628</v>
       </c>
       <c r="J468" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K468" s="2" t="inlineStr">
         <is>
@@ -45456,10 +45456,10 @@
         <v>4822</v>
       </c>
       <c r="I469" s="2" t="n">
-        <v>14466</v>
+        <v>24110</v>
       </c>
       <c r="J469" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K469" s="2" t="inlineStr">
         <is>
@@ -45552,10 +45552,10 @@
         <v>4822</v>
       </c>
       <c r="I470" s="2" t="n">
-        <v>4822</v>
+        <v>14466</v>
       </c>
       <c r="J470" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K470" s="2" t="inlineStr">
         <is>
@@ -45648,10 +45648,10 @@
         <v>4798</v>
       </c>
       <c r="I471" s="2" t="n">
-        <v>52083</v>
+        <v>57155</v>
       </c>
       <c r="J471" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K471" s="2" t="inlineStr">
         <is>
@@ -46416,10 +46416,10 @@
         <v>4703</v>
       </c>
       <c r="I479" s="2" t="n">
-        <v>63589</v>
+        <v>69233</v>
       </c>
       <c r="J479" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K479" s="2" t="inlineStr">
         <is>
@@ -46800,10 +46800,10 @@
         <v>4505</v>
       </c>
       <c r="I483" s="2" t="n">
-        <v>4505</v>
+        <v>13515</v>
       </c>
       <c r="J483" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K483" s="2" t="inlineStr">
         <is>
@@ -47376,10 +47376,10 @@
         <v>4234</v>
       </c>
       <c r="I489" s="2" t="n">
-        <v>17401</v>
+        <v>25869</v>
       </c>
       <c r="J489" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K489" s="2" t="inlineStr">
         <is>
@@ -47472,10 +47472,10 @@
         <v>4047</v>
       </c>
       <c r="I490" s="2" t="n">
-        <v>48480</v>
+        <v>56574</v>
       </c>
       <c r="J490" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K490" s="2" t="inlineStr">
         <is>
@@ -47568,10 +47568,10 @@
         <v>4044</v>
       </c>
       <c r="I491" s="2" t="n">
-        <v>22758</v>
+        <v>27648</v>
       </c>
       <c r="J491" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K491" s="2" t="inlineStr">
         <is>
@@ -47664,10 +47664,10 @@
         <v>3952</v>
       </c>
       <c r="I492" s="2" t="n">
-        <v>41298</v>
+        <v>44854</v>
       </c>
       <c r="J492" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K492" s="2" t="inlineStr">
         <is>
@@ -48240,10 +48240,10 @@
         <v>3927</v>
       </c>
       <c r="I498" s="2" t="n">
-        <v>60340</v>
+        <v>68194</v>
       </c>
       <c r="J498" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K498" s="2" t="inlineStr">
         <is>
@@ -48336,10 +48336,10 @@
         <v>3925</v>
       </c>
       <c r="I499" s="2" t="n">
-        <v>9813</v>
+        <v>13739</v>
       </c>
       <c r="J499" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K499" s="2" t="inlineStr">
         <is>
@@ -48528,10 +48528,10 @@
         <v>3905</v>
       </c>
       <c r="I501" s="2" t="n">
-        <v>3905</v>
+        <v>11715</v>
       </c>
       <c r="J501" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K501" s="2" t="inlineStr">
         <is>
@@ -48624,10 +48624,10 @@
         <v>3879</v>
       </c>
       <c r="I502" s="2" t="n">
-        <v>5624</v>
+        <v>13382</v>
       </c>
       <c r="J502" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K502" s="2" t="inlineStr">
         <is>
@@ -49104,10 +49104,10 @@
         <v>3804</v>
       </c>
       <c r="I507" s="2" t="n">
-        <v>3804</v>
+        <v>11412</v>
       </c>
       <c r="J507" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K507" s="2" t="inlineStr">
         <is>
@@ -49680,10 +49680,10 @@
         <v>3763</v>
       </c>
       <c r="I513" s="2" t="n">
-        <v>26339</v>
+        <v>33865</v>
       </c>
       <c r="J513" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K513" s="2" t="inlineStr">
         <is>
@@ -50064,10 +50064,10 @@
         <v>3736</v>
       </c>
       <c r="I517" s="2" t="n">
-        <v>43298</v>
+        <v>45692</v>
       </c>
       <c r="J517" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K517" s="2" t="inlineStr">
         <is>
@@ -50736,10 +50736,10 @@
         <v>3498</v>
       </c>
       <c r="I524" s="2" t="n">
-        <v>21666</v>
+        <v>28662</v>
       </c>
       <c r="J524" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K524" s="2" t="inlineStr">
         <is>
@@ -50832,10 +50832,10 @@
         <v>3469</v>
       </c>
       <c r="I525" s="2" t="n">
-        <v>19103</v>
+        <v>23533</v>
       </c>
       <c r="J525" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K525" s="2" t="inlineStr">
         <is>
@@ -51216,10 +51216,10 @@
         <v>3392</v>
       </c>
       <c r="I529" s="2" t="n">
-        <v>21469</v>
+        <v>28253</v>
       </c>
       <c r="J529" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K529" s="2" t="inlineStr">
         <is>
@@ -52080,10 +52080,10 @@
         <v>3232</v>
       </c>
       <c r="I538" s="2" t="n">
-        <v>3232</v>
+        <v>9696</v>
       </c>
       <c r="J538" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K538" s="2" t="inlineStr">
         <is>
@@ -52176,10 +52176,10 @@
         <v>3154</v>
       </c>
       <c r="I539" s="2" t="n">
-        <v>52042</v>
+        <v>57956</v>
       </c>
       <c r="J539" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K539" s="2" t="inlineStr">
         <is>
@@ -52368,10 +52368,10 @@
         <v>3103</v>
       </c>
       <c r="I541" s="2" t="n">
-        <v>15323</v>
+        <v>21529</v>
       </c>
       <c r="J541" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K541" s="2" t="inlineStr">
         <is>
@@ -52464,10 +52464,10 @@
         <v>3060</v>
       </c>
       <c r="I542" s="2" t="n">
-        <v>11700</v>
+        <v>17820</v>
       </c>
       <c r="J542" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K542" s="2" t="inlineStr">
         <is>
@@ -53136,10 +53136,10 @@
         <v>2928</v>
       </c>
       <c r="I549" s="2" t="n">
-        <v>25376</v>
+        <v>29280</v>
       </c>
       <c r="J549" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K549" s="2" t="inlineStr">
         <is>
@@ -53712,10 +53712,10 @@
         <v>2898</v>
       </c>
       <c r="I555" s="2" t="n">
-        <v>20147</v>
+        <v>23975</v>
       </c>
       <c r="J555" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K555" s="2" t="inlineStr">
         <is>
@@ -53904,10 +53904,10 @@
         <v>2893</v>
       </c>
       <c r="I557" s="2" t="n">
-        <v>2893</v>
+        <v>8679</v>
       </c>
       <c r="J557" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K557" s="2" t="inlineStr">
         <is>
@@ -54000,10 +54000,10 @@
         <v>2892</v>
       </c>
       <c r="I558" s="2" t="n">
-        <v>24582</v>
+        <v>27474</v>
       </c>
       <c r="J558" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K558" s="2" t="inlineStr">
         <is>
@@ -54480,10 +54480,10 @@
         <v>2869</v>
       </c>
       <c r="I563" s="2" t="n">
-        <v>32115</v>
+        <v>37853</v>
       </c>
       <c r="J563" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K563" s="2" t="inlineStr">
         <is>
@@ -54672,10 +54672,10 @@
         <v>2863</v>
       </c>
       <c r="I565" s="2" t="n">
-        <v>33433</v>
+        <v>39159</v>
       </c>
       <c r="J565" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K565" s="2" t="inlineStr">
         <is>
@@ -54768,10 +54768,10 @@
         <v>2857</v>
       </c>
       <c r="I566" s="2" t="n">
-        <v>30950</v>
+        <v>36664</v>
       </c>
       <c r="J566" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K566" s="2" t="inlineStr">
         <is>
@@ -55632,10 +55632,10 @@
         <v>2822</v>
       </c>
       <c r="I575" s="2" t="n">
-        <v>17871</v>
+        <v>23515</v>
       </c>
       <c r="J575" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K575" s="2" t="inlineStr">
         <is>
@@ -55824,10 +55824,10 @@
         <v>2822</v>
       </c>
       <c r="I577" s="2" t="n">
-        <v>2822</v>
+        <v>8466</v>
       </c>
       <c r="J577" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K577" s="2" t="inlineStr">
         <is>
@@ -55920,10 +55920,10 @@
         <v>2821</v>
       </c>
       <c r="I578" s="2" t="n">
-        <v>46547</v>
+        <v>49369</v>
       </c>
       <c r="J578" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K578" s="2" t="inlineStr">
         <is>
@@ -56304,10 +56304,10 @@
         <v>2730</v>
       </c>
       <c r="I582" s="2" t="n">
-        <v>42514</v>
+        <v>45872</v>
       </c>
       <c r="J582" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K582" s="2" t="inlineStr">
         <is>
@@ -56400,10 +56400,10 @@
         <v>2727</v>
       </c>
       <c r="I583" s="2" t="n">
-        <v>2727</v>
+        <v>8181</v>
       </c>
       <c r="J583" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K583" s="2" t="inlineStr">
         <is>
@@ -57072,10 +57072,10 @@
         <v>2684</v>
       </c>
       <c r="I590" s="2" t="n">
-        <v>17326</v>
+        <v>22694</v>
       </c>
       <c r="J590" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
@@ -57168,10 +57168,10 @@
         <v>2682</v>
       </c>
       <c r="I591" s="2" t="n">
-        <v>2682</v>
+        <v>8046</v>
       </c>
       <c r="J591" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K591" s="2" t="inlineStr">
         <is>
@@ -58032,10 +58032,10 @@
         <v>2446</v>
       </c>
       <c r="I600" s="2" t="n">
-        <v>28141</v>
+        <v>33033</v>
       </c>
       <c r="J600" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
@@ -58128,10 +58128,10 @@
         <v>2441</v>
       </c>
       <c r="I601" s="2" t="n">
-        <v>14646</v>
+        <v>24410</v>
       </c>
       <c r="J601" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K601" s="2" t="inlineStr">
         <is>
@@ -58224,10 +58224,10 @@
         <v>2441</v>
       </c>
       <c r="I602" s="2" t="n">
-        <v>12696</v>
+        <v>17578</v>
       </c>
       <c r="J602" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
@@ -58896,10 +58896,10 @@
         <v>2352</v>
       </c>
       <c r="I609" s="2" t="n">
-        <v>2352</v>
+        <v>7056</v>
       </c>
       <c r="J609" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K609" s="2" t="inlineStr">
         <is>
@@ -58992,10 +58992,10 @@
         <v>2350</v>
       </c>
       <c r="I610" s="2" t="n">
-        <v>7050</v>
+        <v>11750</v>
       </c>
       <c r="J610" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
@@ -59280,10 +59280,10 @@
         <v>2249</v>
       </c>
       <c r="I613" s="2" t="n">
-        <v>14302</v>
+        <v>18800</v>
       </c>
       <c r="J613" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K613" s="2" t="inlineStr">
         <is>
@@ -60144,10 +60144,10 @@
         <v>2096</v>
       </c>
       <c r="I622" s="2" t="n">
-        <v>4590</v>
+        <v>6686</v>
       </c>
       <c r="J622" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K622" s="2" t="inlineStr">
         <is>
@@ -60336,10 +60336,10 @@
         <v>2025</v>
       </c>
       <c r="I624" s="2" t="n">
-        <v>30880</v>
+        <v>33178</v>
       </c>
       <c r="J624" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K624" s="2" t="inlineStr">
         <is>
@@ -60432,10 +60432,10 @@
         <v>2021</v>
       </c>
       <c r="I625" s="2" t="n">
-        <v>2021</v>
+        <v>6063</v>
       </c>
       <c r="J625" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K625" s="2" t="inlineStr">
         <is>
@@ -60528,10 +60528,10 @@
         <v>2014</v>
       </c>
       <c r="I626" s="2" t="n">
-        <v>18151</v>
+        <v>22179</v>
       </c>
       <c r="J626" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K626" s="2" t="inlineStr">
         <is>
@@ -61392,10 +61392,10 @@
         <v>1953</v>
       </c>
       <c r="I635" s="2" t="n">
-        <v>3906</v>
+        <v>7812</v>
       </c>
       <c r="J635" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K635" s="2" t="inlineStr">
         <is>
@@ -61488,10 +61488,10 @@
         <v>1953</v>
       </c>
       <c r="I636" s="2" t="n">
-        <v>15624</v>
+        <v>19530</v>
       </c>
       <c r="J636" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K636" s="2" t="inlineStr">
         <is>
@@ -61776,10 +61776,10 @@
         <v>1940</v>
       </c>
       <c r="I639" s="2" t="n">
-        <v>1940</v>
+        <v>5820</v>
       </c>
       <c r="J639" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K639" s="2" t="inlineStr">
         <is>
@@ -61968,10 +61968,10 @@
         <v>1928</v>
       </c>
       <c r="I641" s="2" t="n">
-        <v>1928</v>
+        <v>5784</v>
       </c>
       <c r="J641" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K641" s="2" t="inlineStr">
         <is>
@@ -62448,10 +62448,10 @@
         <v>1916</v>
       </c>
       <c r="I646" s="2" t="n">
-        <v>1916</v>
+        <v>5748</v>
       </c>
       <c r="J646" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K646" s="2" t="inlineStr">
         <is>
@@ -63024,10 +63024,10 @@
         <v>1881</v>
       </c>
       <c r="I652" s="2" t="n">
-        <v>31977</v>
+        <v>35739</v>
       </c>
       <c r="J652" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K652" s="2" t="inlineStr">
         <is>
@@ -63408,10 +63408,10 @@
         <v>1873</v>
       </c>
       <c r="I656" s="2" t="n">
-        <v>1873</v>
+        <v>5619</v>
       </c>
       <c r="J656" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K656" s="2" t="inlineStr">
         <is>
@@ -63696,10 +63696,10 @@
         <v>1849</v>
       </c>
       <c r="I659" s="2" t="n">
-        <v>11607</v>
+        <v>15305</v>
       </c>
       <c r="J659" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K659" s="2" t="inlineStr">
         <is>
@@ -64752,10 +64752,10 @@
         <v>1739</v>
       </c>
       <c r="I670" s="2" t="n">
-        <v>13584</v>
+        <v>16406</v>
       </c>
       <c r="J670" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K670" s="2" t="inlineStr">
         <is>
@@ -65136,10 +65136,10 @@
         <v>1671</v>
       </c>
       <c r="I674" s="2" t="n">
-        <v>1671</v>
+        <v>5013</v>
       </c>
       <c r="J674" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K674" s="2" t="inlineStr">
         <is>
@@ -65328,10 +65328,10 @@
         <v>1652</v>
       </c>
       <c r="I676" s="2" t="n">
-        <v>10325</v>
+        <v>13629</v>
       </c>
       <c r="J676" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K676" s="2" t="inlineStr">
         <is>
@@ -66096,10 +66096,10 @@
         <v>1575</v>
       </c>
       <c r="I684" s="2" t="n">
-        <v>1575</v>
+        <v>4725</v>
       </c>
       <c r="J684" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K684" s="2" t="inlineStr">
         <is>
@@ -66288,10 +66288,10 @@
         <v>1552</v>
       </c>
       <c r="I686" s="2" t="n">
-        <v>13435</v>
+        <v>15473</v>
       </c>
       <c r="J686" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K686" s="2" t="inlineStr">
         <is>
@@ -66384,10 +66384,10 @@
         <v>1539</v>
       </c>
       <c r="I687" s="2" t="n">
-        <v>10296</v>
+        <v>13374</v>
       </c>
       <c r="J687" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K687" s="2" t="inlineStr">
         <is>
@@ -66480,10 +66480,10 @@
         <v>1536</v>
       </c>
       <c r="I688" s="2" t="n">
-        <v>13127</v>
+        <v>15611</v>
       </c>
       <c r="J688" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K688" s="2" t="inlineStr">
         <is>
@@ -66672,10 +66672,10 @@
         <v>1530</v>
       </c>
       <c r="I690" s="2" t="n">
-        <v>1530</v>
+        <v>4590</v>
       </c>
       <c r="J690" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K690" s="2" t="inlineStr">
         <is>
@@ -66864,10 +66864,10 @@
         <v>1524</v>
       </c>
       <c r="I692" s="2" t="n">
-        <v>1524</v>
+        <v>4572</v>
       </c>
       <c r="J692" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K692" s="2" t="inlineStr">
         <is>
@@ -67056,10 +67056,10 @@
         <v>1504</v>
       </c>
       <c r="I694" s="2" t="n">
-        <v>10295</v>
+        <v>13303</v>
       </c>
       <c r="J694" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K694" s="2" t="inlineStr">
         <is>
@@ -67344,10 +67344,10 @@
         <v>1455</v>
       </c>
       <c r="I697" s="2" t="n">
-        <v>1455</v>
+        <v>4365</v>
       </c>
       <c r="J697" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K697" s="2" t="inlineStr">
         <is>
@@ -67440,10 +67440,10 @@
         <v>1448</v>
       </c>
       <c r="I698" s="2" t="n">
-        <v>1448</v>
+        <v>4344</v>
       </c>
       <c r="J698" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K698" s="2" t="inlineStr">
         <is>
@@ -67536,10 +67536,10 @@
         <v>1440</v>
       </c>
       <c r="I699" s="2" t="n">
-        <v>9900</v>
+        <v>12780</v>
       </c>
       <c r="J699" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K699" s="2" t="inlineStr">
         <is>
@@ -67824,10 +67824,10 @@
         <v>1411</v>
       </c>
       <c r="I702" s="2" t="n">
-        <v>1411</v>
+        <v>4233</v>
       </c>
       <c r="J702" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K702" s="2" t="inlineStr">
         <is>
@@ -68112,10 +68112,10 @@
         <v>1368</v>
       </c>
       <c r="I705" s="2" t="n">
-        <v>1368</v>
+        <v>4104</v>
       </c>
       <c r="J705" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K705" s="2" t="inlineStr">
         <is>
@@ -68400,10 +68400,10 @@
         <v>1310</v>
       </c>
       <c r="I708" s="2" t="n">
-        <v>3930</v>
+        <v>6550</v>
       </c>
       <c r="J708" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K708" s="2" t="inlineStr">
         <is>
@@ -68784,10 +68784,10 @@
         <v>1259</v>
       </c>
       <c r="I712" s="2" t="n">
-        <v>1259</v>
+        <v>6295</v>
       </c>
       <c r="J712" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K712" s="2" t="inlineStr">
         <is>
@@ -69168,10 +69168,10 @@
         <v>1161</v>
       </c>
       <c r="I716" s="2" t="n">
-        <v>1161</v>
+        <v>3483</v>
       </c>
       <c r="J716" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K716" s="2" t="inlineStr">
         <is>
@@ -69264,10 +69264,10 @@
         <v>1156</v>
       </c>
       <c r="I717" s="2" t="n">
-        <v>8625</v>
+        <v>10937</v>
       </c>
       <c r="J717" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K717" s="2" t="inlineStr">
         <is>
@@ -69360,10 +69360,10 @@
         <v>1156</v>
       </c>
       <c r="I718" s="2" t="n">
-        <v>3424</v>
+        <v>5648</v>
       </c>
       <c r="J718" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K718" s="2" t="inlineStr">
         <is>
@@ -69552,10 +69552,10 @@
         <v>1080</v>
       </c>
       <c r="I720" s="2" t="n">
-        <v>4320</v>
+        <v>6480</v>
       </c>
       <c r="J720" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K720" s="2" t="inlineStr">
         <is>
@@ -69936,10 +69936,10 @@
         <v>1031</v>
       </c>
       <c r="I724" s="2" t="n">
-        <v>1031</v>
+        <v>3093</v>
       </c>
       <c r="J724" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K724" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: Daily payout audit & Non-SEBI ledger update [2026-09-05]
</commit_message>
<xml_diff>
--- a/reports/telegram_sebi_10day_report.xlsx
+++ b/reports/telegram_sebi_10day_report.xlsx
@@ -624,10 +624,10 @@
         <v>569271</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>10053704</v>
+        <v>10180884</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -720,10 +720,10 @@
         <v>495829</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>3332810</v>
+        <v>3430960</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -816,10 +816,10 @@
         <v>393135</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1315454</v>
+        <v>1379177</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -1008,10 +1008,10 @@
         <v>211523</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1579551</v>
+        <v>1647254</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -1104,10 +1104,10 @@
         <v>195176</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1020479</v>
+        <v>1215655</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -1200,10 +1200,10 @@
         <v>162819</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>3310240</v>
+        <v>3428391</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -1296,10 +1296,10 @@
         <v>158965</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1027797</v>
+        <v>1036262</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1392,10 +1392,10 @@
         <v>151478</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>2394725</v>
+        <v>2477367</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1488,10 +1488,10 @@
         <v>146807</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>2381906</v>
+        <v>2528713</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1680,10 +1680,10 @@
         <v>136719</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1530758</v>
+        <v>1603546</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1776,10 +1776,10 @@
         <v>127846</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>1416254</v>
+        <v>1450807</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1872,10 +1872,10 @@
         <v>114194</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>782507</v>
+        <v>793556</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -1968,10 +1968,10 @@
         <v>107479</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1423081</v>
+        <v>1456077</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -2064,10 +2064,10 @@
         <v>106625</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>912956</v>
+        <v>922772</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -2256,10 +2256,10 @@
         <v>102168</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>856754</v>
+        <v>915338</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -2352,10 +2352,10 @@
         <v>99486</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1698808</v>
+        <v>1747459</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
@@ -2544,10 +2544,10 @@
         <v>94169</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1847031</v>
+        <v>1903903</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -2736,10 +2736,10 @@
         <v>88046</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1152770</v>
+        <v>1173843</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -2928,10 +2928,10 @@
         <v>82493</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>372214</v>
+        <v>391624</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -3024,10 +3024,10 @@
         <v>80760</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>760780</v>
+        <v>770680</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -3312,10 +3312,10 @@
         <v>78026</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>164563</v>
+        <v>242589</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -3408,10 +3408,10 @@
         <v>76419</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>1100498</v>
+        <v>1162242</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
@@ -3504,10 +3504,10 @@
         <v>75133</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>673214</v>
+        <v>732412</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -3600,10 +3600,10 @@
         <v>74332</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>835167</v>
+        <v>854578</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
@@ -3696,10 +3696,10 @@
         <v>70572</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>633613</v>
+        <v>704185</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -3792,10 +3792,10 @@
         <v>69504</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>764702</v>
+        <v>787600</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -3888,10 +3888,10 @@
         <v>68460</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>332289</v>
+        <v>341991</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -3984,10 +3984,10 @@
         <v>68202</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>484119</v>
+        <v>497380</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
@@ -4080,10 +4080,10 @@
         <v>66718</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>912167</v>
+        <v>955891</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -4176,10 +4176,10 @@
         <v>66703</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>588457</v>
+        <v>636125</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -4272,10 +4272,10 @@
         <v>65645</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>764473</v>
+        <v>830118</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>65193</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>735875</v>
+        <v>745230</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -4464,10 +4464,10 @@
         <v>65111</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>894190</v>
+        <v>938562</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -4656,10 +4656,10 @@
         <v>63293</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>634931</v>
+        <v>698224</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -4752,10 +4752,10 @@
         <v>60916</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>403618</v>
+        <v>464534</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -4848,10 +4848,10 @@
         <v>60291</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>945131</v>
+        <v>1005422</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -5040,10 +5040,10 @@
         <v>58176</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>655952</v>
+        <v>690221</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -5232,10 +5232,10 @@
         <v>57276</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>539420</v>
+        <v>575750</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -5328,10 +5328,10 @@
         <v>56775</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>777866</v>
+        <v>834641</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -5712,10 +5712,10 @@
         <v>54993</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>731863</v>
+        <v>768699</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -5808,10 +5808,10 @@
         <v>54825</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>702264</v>
+        <v>725075</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -5904,10 +5904,10 @@
         <v>53890</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>1155910</v>
+        <v>1170608</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -6192,10 +6192,10 @@
         <v>52868</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>105736</v>
+        <v>158604</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
@@ -6288,10 +6288,10 @@
         <v>51138</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>605944</v>
+        <v>643668</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -6384,10 +6384,10 @@
         <v>50870</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>381579</v>
+        <v>394111</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
@@ -6576,10 +6576,10 @@
         <v>48785</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>950169</v>
+        <v>988231</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
@@ -6672,10 +6672,10 @@
         <v>48595</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>251126</v>
+        <v>299721</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -6960,10 +6960,10 @@
         <v>48086</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>838867</v>
+        <v>884554</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
@@ -7056,10 +7056,10 @@
         <v>47876</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>713083</v>
+        <v>741150</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
@@ -7248,10 +7248,10 @@
         <v>45340</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>310220</v>
+        <v>355560</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
@@ -7344,10 +7344,10 @@
         <v>43416</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>137472</v>
+        <v>140479</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
@@ -7440,10 +7440,10 @@
         <v>43047</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>562203</v>
+        <v>579341</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
@@ -7536,10 +7536,10 @@
         <v>42572</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>442075</v>
+        <v>453638</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
@@ -7728,10 +7728,10 @@
         <v>42172</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>359942</v>
+        <v>402114</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
@@ -7920,10 +7920,10 @@
         <v>41270</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>207191</v>
+        <v>222555</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
@@ -8016,10 +8016,10 @@
         <v>40719</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>648150</v>
+        <v>654886</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
@@ -8112,10 +8112,10 @@
         <v>39334</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>472762</v>
+        <v>494593</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
@@ -8208,10 +8208,10 @@
         <v>39288</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>586453</v>
+        <v>609842</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
@@ -8304,10 +8304,10 @@
         <v>39193</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>187937</v>
+        <v>193814</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
@@ -8400,10 +8400,10 @@
         <v>39173</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>564197</v>
+        <v>573230</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
@@ -8496,10 +8496,10 @@
         <v>38879</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>97282</v>
+        <v>136161</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
@@ -8592,10 +8592,10 @@
         <v>38479</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>721336</v>
+        <v>731084</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
@@ -8880,10 +8880,10 @@
         <v>37610</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>478530</v>
+        <v>483328</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
@@ -9072,10 +9072,10 @@
         <v>37246</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>233121</v>
+        <v>241331</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -9168,10 +9168,10 @@
         <v>37064</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>117782</v>
+        <v>154846</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
@@ -9360,10 +9360,10 @@
         <v>36417</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>411872</v>
+        <v>421658</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
@@ -9456,10 +9456,10 @@
         <v>35954</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>185552</v>
+        <v>198967</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -9552,10 +9552,10 @@
         <v>35835</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>548891</v>
+        <v>567749</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
@@ -9648,10 +9648,10 @@
         <v>35080</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>477332</v>
+        <v>487583</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
@@ -9744,10 +9744,10 @@
         <v>34616</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>101871</v>
+        <v>105025</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
@@ -9840,10 +9840,10 @@
         <v>34370</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>567258</v>
+        <v>584935</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
@@ -9936,10 +9936,10 @@
         <v>34334</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>398836</v>
+        <v>415401</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
@@ -10032,10 +10032,10 @@
         <v>33783</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>505202</v>
+        <v>516584</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K100" s="2" t="inlineStr">
         <is>
@@ -10128,10 +10128,10 @@
         <v>33544</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>564223</v>
+        <v>578570</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
@@ -10224,10 +10224,10 @@
         <v>33294</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>245162</v>
+        <v>259404</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
@@ -10320,10 +10320,10 @@
         <v>33238</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>192221</v>
+        <v>201340</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
@@ -10416,10 +10416,10 @@
         <v>33182</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>204115</v>
+        <v>237297</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
@@ -10512,10 +10512,10 @@
         <v>33063</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>554292</v>
+        <v>576611</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
@@ -10608,10 +10608,10 @@
         <v>32476</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>250055</v>
+        <v>257128</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K106" s="2" t="inlineStr">
         <is>
@@ -10992,10 +10992,10 @@
         <v>31199</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>363247</v>
+        <v>377330</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
@@ -11088,10 +11088,10 @@
         <v>31103</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>290427</v>
+        <v>321530</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
@@ -11184,10 +11184,10 @@
         <v>30867</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>170052</v>
+        <v>173934</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
@@ -11280,10 +11280,10 @@
         <v>30716</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>303065</v>
+        <v>315633</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
@@ -11376,10 +11376,10 @@
         <v>30528</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>327435</v>
+        <v>357963</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
@@ -11472,10 +11472,10 @@
         <v>30200</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>111204</v>
+        <v>118730</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K115" s="2" t="inlineStr">
         <is>
@@ -11760,10 +11760,10 @@
         <v>29222</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>315613</v>
+        <v>326717</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K118" s="2" t="inlineStr">
         <is>
@@ -11952,10 +11952,10 @@
         <v>28689</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>306748</v>
+        <v>316272</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K120" s="2" t="inlineStr">
         <is>
@@ -12048,10 +12048,10 @@
         <v>28592</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>384715</v>
+        <v>413307</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K121" s="2" t="inlineStr">
         <is>
@@ -12144,10 +12144,10 @@
         <v>28319</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>329713</v>
+        <v>349463</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K122" s="2" t="inlineStr">
         <is>
@@ -12240,10 +12240,10 @@
         <v>28151</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>210775</v>
+        <v>216589</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K123" s="2" t="inlineStr">
         <is>
@@ -12624,10 +12624,10 @@
         <v>27646</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>301202</v>
+        <v>322860</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
@@ -12720,10 +12720,10 @@
         <v>27571</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>236285</v>
+        <v>240849</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K128" s="2" t="inlineStr">
         <is>
@@ -12816,10 +12816,10 @@
         <v>27501</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>298407</v>
+        <v>321399</v>
       </c>
       <c r="J129" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K129" s="2" t="inlineStr">
         <is>
@@ -12912,10 +12912,10 @@
         <v>27418</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>188445</v>
+        <v>215863</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
@@ -13008,10 +13008,10 @@
         <v>27294</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>382138</v>
+        <v>403612</v>
       </c>
       <c r="J131" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
@@ -13200,10 +13200,10 @@
         <v>26996</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>208385</v>
+        <v>212460</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K133" s="2" t="inlineStr">
         <is>
@@ -13296,10 +13296,10 @@
         <v>26814</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>382876</v>
+        <v>398006</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K134" s="2" t="inlineStr">
         <is>
@@ -13488,10 +13488,10 @@
         <v>26348</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>351941</v>
+        <v>365115</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K136" s="2" t="inlineStr">
         <is>
@@ -13584,10 +13584,10 @@
         <v>26303</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>165180</v>
+        <v>191483</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K137" s="2" t="inlineStr">
         <is>
@@ -13776,10 +13776,10 @@
         <v>26168</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>366459</v>
+        <v>369370</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K139" s="2" t="inlineStr">
         <is>
@@ -13872,10 +13872,10 @@
         <v>26042</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>143714</v>
+        <v>148536</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K140" s="2" t="inlineStr">
         <is>
@@ -14064,10 +14064,10 @@
         <v>25401</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>290314</v>
+        <v>297463</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
@@ -14160,10 +14160,10 @@
         <v>25381</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>270896</v>
+        <v>286514</v>
       </c>
       <c r="J143" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
@@ -14256,10 +14256,10 @@
         <v>25182</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>114710</v>
+        <v>139892</v>
       </c>
       <c r="J144" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
@@ -14352,10 +14352,10 @@
         <v>25120</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>387549</v>
+        <v>407510</v>
       </c>
       <c r="J145" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K145" s="2" t="inlineStr">
         <is>
@@ -14448,10 +14448,10 @@
         <v>25014</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>149777</v>
+        <v>174791</v>
       </c>
       <c r="J146" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K146" s="2" t="inlineStr">
         <is>
@@ -14544,10 +14544,10 @@
         <v>24560</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>172828</v>
+        <v>197388</v>
       </c>
       <c r="J147" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K147" s="2" t="inlineStr">
         <is>
@@ -14640,10 +14640,10 @@
         <v>24466</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>329982</v>
+        <v>348637</v>
       </c>
       <c r="J148" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K148" s="2" t="inlineStr">
         <is>
@@ -14736,10 +14736,10 @@
         <v>24370</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>342219</v>
+        <v>343646</v>
       </c>
       <c r="J149" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K149" s="2" t="inlineStr">
         <is>
@@ -14832,10 +14832,10 @@
         <v>24263</v>
       </c>
       <c r="I150" s="2" t="n">
-        <v>65018</v>
+        <v>89281</v>
       </c>
       <c r="J150" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K150" s="2" t="inlineStr">
         <is>
@@ -14928,10 +14928,10 @@
         <v>23733</v>
       </c>
       <c r="I151" s="2" t="n">
-        <v>89006</v>
+        <v>99344</v>
       </c>
       <c r="J151" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K151" s="2" t="inlineStr">
         <is>
@@ -15120,10 +15120,10 @@
         <v>23148</v>
       </c>
       <c r="I153" s="2" t="n">
-        <v>143466</v>
+        <v>166614</v>
       </c>
       <c r="J153" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K153" s="2" t="inlineStr">
         <is>
@@ -15216,10 +15216,10 @@
         <v>23055</v>
       </c>
       <c r="I154" s="2" t="n">
-        <v>225280</v>
+        <v>238454</v>
       </c>
       <c r="J154" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
@@ -15408,10 +15408,10 @@
         <v>22576</v>
       </c>
       <c r="I156" s="2" t="n">
-        <v>350596</v>
+        <v>371950</v>
       </c>
       <c r="J156" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
@@ -15504,10 +15504,10 @@
         <v>22114</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>191154</v>
+        <v>212543</v>
       </c>
       <c r="J157" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
@@ -15600,10 +15600,10 @@
         <v>21731</v>
       </c>
       <c r="I158" s="2" t="n">
-        <v>293780</v>
+        <v>305114</v>
       </c>
       <c r="J158" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K158" s="2" t="inlineStr">
         <is>
@@ -15792,10 +15792,10 @@
         <v>21447</v>
       </c>
       <c r="I160" s="2" t="n">
-        <v>218501</v>
+        <v>239815</v>
       </c>
       <c r="J160" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K160" s="2" t="inlineStr">
         <is>
@@ -15888,10 +15888,10 @@
         <v>21410</v>
       </c>
       <c r="I161" s="2" t="n">
-        <v>320664</v>
+        <v>327009</v>
       </c>
       <c r="J161" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K161" s="2" t="inlineStr">
         <is>
@@ -15984,10 +15984,10 @@
         <v>21393</v>
       </c>
       <c r="I162" s="2" t="n">
-        <v>239850</v>
+        <v>245903</v>
       </c>
       <c r="J162" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
@@ -16176,10 +16176,10 @@
         <v>21350</v>
       </c>
       <c r="I164" s="2" t="n">
-        <v>190115</v>
+        <v>200277</v>
       </c>
       <c r="J164" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K164" s="2" t="inlineStr">
         <is>
@@ -16272,10 +16272,10 @@
         <v>21292</v>
       </c>
       <c r="I165" s="2" t="n">
-        <v>281974</v>
+        <v>296055</v>
       </c>
       <c r="J165" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K165" s="2" t="inlineStr">
         <is>
@@ -16464,10 +16464,10 @@
         <v>21056</v>
       </c>
       <c r="I167" s="2" t="n">
-        <v>224768</v>
+        <v>228675</v>
       </c>
       <c r="J167" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K167" s="2" t="inlineStr">
         <is>
@@ -16560,10 +16560,10 @@
         <v>20991</v>
       </c>
       <c r="I168" s="2" t="n">
-        <v>192300</v>
+        <v>199133</v>
       </c>
       <c r="J168" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K168" s="2" t="inlineStr">
         <is>
@@ -16656,10 +16656,10 @@
         <v>20486</v>
       </c>
       <c r="I169" s="2" t="n">
-        <v>168816</v>
+        <v>189302</v>
       </c>
       <c r="J169" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K169" s="2" t="inlineStr">
         <is>
@@ -16848,10 +16848,10 @@
         <v>20077</v>
       </c>
       <c r="I171" s="2" t="n">
-        <v>40154</v>
+        <v>60231</v>
       </c>
       <c r="J171" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K171" s="2" t="inlineStr">
         <is>
@@ -16944,10 +16944,10 @@
         <v>20067</v>
       </c>
       <c r="I172" s="2" t="n">
-        <v>137224</v>
+        <v>146062</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
@@ -17328,10 +17328,10 @@
         <v>19651</v>
       </c>
       <c r="I176" s="2" t="n">
-        <v>211838</v>
+        <v>227559</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
@@ -17616,10 +17616,10 @@
         <v>19421</v>
       </c>
       <c r="I179" s="2" t="n">
-        <v>108730</v>
+        <v>124253</v>
       </c>
       <c r="J179" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K179" s="2" t="inlineStr">
         <is>
@@ -18000,10 +18000,10 @@
         <v>19326</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>114406</v>
+        <v>117968</v>
       </c>
       <c r="J183" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K183" s="2" t="inlineStr">
         <is>
@@ -18096,10 +18096,10 @@
         <v>19271</v>
       </c>
       <c r="I184" s="2" t="n">
-        <v>161913</v>
+        <v>167699</v>
       </c>
       <c r="J184" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K184" s="2" t="inlineStr">
         <is>
@@ -18192,10 +18192,10 @@
         <v>19255</v>
       </c>
       <c r="I185" s="2" t="n">
-        <v>253615</v>
+        <v>272870</v>
       </c>
       <c r="J185" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K185" s="2" t="inlineStr">
         <is>
@@ -18576,10 +18576,10 @@
         <v>19075</v>
       </c>
       <c r="I189" s="2" t="n">
-        <v>264882</v>
+        <v>281978</v>
       </c>
       <c r="J189" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K189" s="2" t="inlineStr">
         <is>
@@ -18768,10 +18768,10 @@
         <v>18820</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>100876</v>
+        <v>113674</v>
       </c>
       <c r="J191" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K191" s="2" t="inlineStr">
         <is>
@@ -18864,10 +18864,10 @@
         <v>18691</v>
       </c>
       <c r="I192" s="2" t="n">
-        <v>146941</v>
+        <v>151638</v>
       </c>
       <c r="J192" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
@@ -18960,10 +18960,10 @@
         <v>18578</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>284724</v>
+        <v>288677</v>
       </c>
       <c r="J193" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
@@ -19056,10 +19056,10 @@
         <v>18517</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>205161</v>
+        <v>222666</v>
       </c>
       <c r="J194" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
@@ -19248,10 +19248,10 @@
         <v>18440</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>114042</v>
+        <v>132482</v>
       </c>
       <c r="J196" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
@@ -19344,10 +19344,10 @@
         <v>18435</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>217204</v>
+        <v>223996</v>
       </c>
       <c r="J197" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K197" s="2" t="inlineStr">
         <is>
@@ -19536,10 +19536,10 @@
         <v>18146</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>78078</v>
+        <v>86896</v>
       </c>
       <c r="J199" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K199" s="2" t="inlineStr">
         <is>
@@ -19824,10 +19824,10 @@
         <v>17842</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>278455</v>
+        <v>284668</v>
       </c>
       <c r="J202" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
@@ -19920,10 +19920,10 @@
         <v>17796</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>245106</v>
+        <v>254149</v>
       </c>
       <c r="J203" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
@@ -20016,10 +20016,10 @@
         <v>17782</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>163872</v>
+        <v>180116</v>
       </c>
       <c r="J204" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
@@ -20304,10 +20304,10 @@
         <v>17625</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>107502</v>
+        <v>111419</v>
       </c>
       <c r="J207" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
@@ -20400,10 +20400,10 @@
         <v>17525</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>172220</v>
+        <v>187772</v>
       </c>
       <c r="J208" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K208" s="2" t="inlineStr">
         <is>
@@ -20688,10 +20688,10 @@
         <v>17287</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>188566</v>
+        <v>197386</v>
       </c>
       <c r="J211" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K211" s="2" t="inlineStr">
         <is>
@@ -20784,10 +20784,10 @@
         <v>17124</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>217376</v>
+        <v>234500</v>
       </c>
       <c r="J212" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K212" s="2" t="inlineStr">
         <is>
@@ -20880,10 +20880,10 @@
         <v>17025</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>264086</v>
+        <v>272657</v>
       </c>
       <c r="J213" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K213" s="2" t="inlineStr">
         <is>
@@ -21168,10 +21168,10 @@
         <v>16821</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>129625</v>
+        <v>132670</v>
       </c>
       <c r="J216" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
@@ -21264,10 +21264,10 @@
         <v>16622</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>33244</v>
+        <v>49866</v>
       </c>
       <c r="J217" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K217" s="2" t="inlineStr">
         <is>
@@ -21456,10 +21456,10 @@
         <v>16587</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>189848</v>
+        <v>198652</v>
       </c>
       <c r="J219" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
@@ -21552,10 +21552,10 @@
         <v>16561</v>
       </c>
       <c r="I220" s="2" t="n">
-        <v>305363</v>
+        <v>314982</v>
       </c>
       <c r="J220" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
@@ -21744,10 +21744,10 @@
         <v>16494</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>152305</v>
+        <v>154421</v>
       </c>
       <c r="J222" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K222" s="2" t="inlineStr">
         <is>
@@ -22032,10 +22032,10 @@
         <v>16166</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>226592</v>
+        <v>238637</v>
       </c>
       <c r="J225" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
@@ -22128,10 +22128,10 @@
         <v>16126</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>193317</v>
+        <v>197463</v>
       </c>
       <c r="J226" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K226" s="2" t="inlineStr">
         <is>
@@ -22224,10 +22224,10 @@
         <v>16043</v>
       </c>
       <c r="I227" s="2" t="n">
-        <v>155789</v>
+        <v>163990</v>
       </c>
       <c r="J227" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K227" s="2" t="inlineStr">
         <is>
@@ -22416,10 +22416,10 @@
         <v>15947</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>204174</v>
+        <v>220121</v>
       </c>
       <c r="J229" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K229" s="2" t="inlineStr">
         <is>
@@ -22512,10 +22512,10 @@
         <v>15938</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>189222</v>
+        <v>196604</v>
       </c>
       <c r="J230" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K230" s="2" t="inlineStr">
         <is>
@@ -22608,10 +22608,10 @@
         <v>15807</v>
       </c>
       <c r="I231" s="2" t="n">
-        <v>252207</v>
+        <v>256041</v>
       </c>
       <c r="J231" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K231" s="2" t="inlineStr">
         <is>
@@ -22800,10 +22800,10 @@
         <v>15606</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>92125</v>
+        <v>107731</v>
       </c>
       <c r="J233" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K233" s="2" t="inlineStr">
         <is>
@@ -22896,10 +22896,10 @@
         <v>15532</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>128792</v>
+        <v>144324</v>
       </c>
       <c r="J234" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K234" s="2" t="inlineStr">
         <is>
@@ -23088,10 +23088,10 @@
         <v>15488</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>168348</v>
+        <v>183836</v>
       </c>
       <c r="J236" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
@@ -23280,10 +23280,10 @@
         <v>15275</v>
       </c>
       <c r="I238" s="2" t="n">
-        <v>125404</v>
+        <v>130226</v>
       </c>
       <c r="J238" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K238" s="2" t="inlineStr">
         <is>
@@ -23472,10 +23472,10 @@
         <v>14953</v>
       </c>
       <c r="I240" s="2" t="n">
-        <v>143115</v>
+        <v>147345</v>
       </c>
       <c r="J240" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K240" s="2" t="inlineStr">
         <is>
@@ -23568,10 +23568,10 @@
         <v>14915</v>
       </c>
       <c r="I241" s="2" t="n">
-        <v>169586</v>
+        <v>171364</v>
       </c>
       <c r="J241" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K241" s="2" t="inlineStr">
         <is>
@@ -23760,10 +23760,10 @@
         <v>14654</v>
       </c>
       <c r="I243" s="2" t="n">
-        <v>29308</v>
+        <v>43962</v>
       </c>
       <c r="J243" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K243" s="2" t="inlineStr">
         <is>
@@ -23856,10 +23856,10 @@
         <v>14646</v>
       </c>
       <c r="I244" s="2" t="n">
-        <v>148343</v>
+        <v>152249</v>
       </c>
       <c r="J244" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K244" s="2" t="inlineStr">
         <is>
@@ -24240,10 +24240,10 @@
         <v>14381</v>
       </c>
       <c r="I248" s="2" t="n">
-        <v>90521</v>
+        <v>93938</v>
       </c>
       <c r="J248" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K248" s="2" t="inlineStr">
         <is>
@@ -24432,10 +24432,10 @@
         <v>14380</v>
       </c>
       <c r="I250" s="2" t="n">
-        <v>81240</v>
+        <v>83521</v>
       </c>
       <c r="J250" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K250" s="2" t="inlineStr">
         <is>
@@ -24528,10 +24528,10 @@
         <v>14313</v>
       </c>
       <c r="I251" s="2" t="n">
-        <v>205325</v>
+        <v>208222</v>
       </c>
       <c r="J251" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K251" s="2" t="inlineStr">
         <is>
@@ -24624,10 +24624,10 @@
         <v>14313</v>
       </c>
       <c r="I252" s="2" t="n">
-        <v>113926</v>
+        <v>119633</v>
       </c>
       <c r="J252" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K252" s="2" t="inlineStr">
         <is>
@@ -24816,10 +24816,10 @@
         <v>14158</v>
       </c>
       <c r="I254" s="2" t="n">
-        <v>76058</v>
+        <v>77571</v>
       </c>
       <c r="J254" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K254" s="2" t="inlineStr">
         <is>
@@ -25200,10 +25200,10 @@
         <v>14114</v>
       </c>
       <c r="I258" s="2" t="n">
-        <v>28228</v>
+        <v>42342</v>
       </c>
       <c r="J258" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K258" s="2" t="inlineStr">
         <is>
@@ -25392,10 +25392,10 @@
         <v>14097</v>
       </c>
       <c r="I260" s="2" t="n">
-        <v>772064</v>
+        <v>774421</v>
       </c>
       <c r="J260" s="2" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K260" s="2" t="inlineStr">
         <is>
@@ -25488,10 +25488,10 @@
         <v>14042</v>
       </c>
       <c r="I261" s="2" t="n">
-        <v>137877</v>
+        <v>140823</v>
       </c>
       <c r="J261" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K261" s="2" t="inlineStr">
         <is>
@@ -25584,10 +25584,10 @@
         <v>13943</v>
       </c>
       <c r="I262" s="2" t="n">
-        <v>255210</v>
+        <v>264549</v>
       </c>
       <c r="J262" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K262" s="2" t="inlineStr">
         <is>
@@ -25776,10 +25776,10 @@
         <v>13860</v>
       </c>
       <c r="I264" s="2" t="n">
-        <v>60504</v>
+        <v>63042</v>
       </c>
       <c r="J264" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K264" s="2" t="inlineStr">
         <is>
@@ -25968,10 +25968,10 @@
         <v>13768</v>
       </c>
       <c r="I266" s="2" t="n">
-        <v>66585</v>
+        <v>69734</v>
       </c>
       <c r="J266" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K266" s="2" t="inlineStr">
         <is>
@@ -26064,10 +26064,10 @@
         <v>13563</v>
       </c>
       <c r="I267" s="2" t="n">
-        <v>139999</v>
+        <v>149763</v>
       </c>
       <c r="J267" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K267" s="2" t="inlineStr">
         <is>
@@ -26160,10 +26160,10 @@
         <v>13541</v>
       </c>
       <c r="I268" s="2" t="n">
-        <v>187225</v>
+        <v>190798</v>
       </c>
       <c r="J268" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K268" s="2" t="inlineStr">
         <is>
@@ -26544,10 +26544,10 @@
         <v>13233</v>
       </c>
       <c r="I272" s="2" t="n">
-        <v>134099</v>
+        <v>137432</v>
       </c>
       <c r="J272" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K272" s="2" t="inlineStr">
         <is>
@@ -26736,10 +26736,10 @@
         <v>13101</v>
       </c>
       <c r="I274" s="2" t="n">
-        <v>28422</v>
+        <v>41523</v>
       </c>
       <c r="J274" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K274" s="2" t="inlineStr">
         <is>
@@ -26832,10 +26832,10 @@
         <v>12786</v>
       </c>
       <c r="I275" s="2" t="n">
-        <v>159287</v>
+        <v>166172</v>
       </c>
       <c r="J275" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K275" s="2" t="inlineStr">
         <is>
@@ -26928,10 +26928,10 @@
         <v>12745</v>
       </c>
       <c r="I276" s="2" t="n">
-        <v>109245</v>
+        <v>110628</v>
       </c>
       <c r="J276" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K276" s="2" t="inlineStr">
         <is>
@@ -27120,10 +27120,10 @@
         <v>12689</v>
       </c>
       <c r="I278" s="2" t="n">
-        <v>141476</v>
+        <v>142913</v>
       </c>
       <c r="J278" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K278" s="2" t="inlineStr">
         <is>
@@ -27216,10 +27216,10 @@
         <v>12600</v>
       </c>
       <c r="I279" s="2" t="n">
-        <v>60480</v>
+        <v>73080</v>
       </c>
       <c r="J279" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K279" s="2" t="inlineStr">
         <is>
@@ -27408,10 +27408,10 @@
         <v>12340</v>
       </c>
       <c r="I281" s="2" t="n">
-        <v>127338</v>
+        <v>131451</v>
       </c>
       <c r="J281" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K281" s="2" t="inlineStr">
         <is>
@@ -27504,10 +27504,10 @@
         <v>12303</v>
       </c>
       <c r="I282" s="2" t="n">
-        <v>211129</v>
+        <v>221488</v>
       </c>
       <c r="J282" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K282" s="2" t="inlineStr">
         <is>
@@ -27792,10 +27792,10 @@
         <v>12058</v>
       </c>
       <c r="I285" s="2" t="n">
-        <v>146139</v>
+        <v>158197</v>
       </c>
       <c r="J285" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K285" s="2" t="inlineStr">
         <is>
@@ -27888,10 +27888,10 @@
         <v>11974</v>
       </c>
       <c r="I286" s="2" t="n">
-        <v>199704</v>
+        <v>207062</v>
       </c>
       <c r="J286" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K286" s="2" t="inlineStr">
         <is>
@@ -28080,10 +28080,10 @@
         <v>11619</v>
       </c>
       <c r="I288" s="2" t="n">
-        <v>157849</v>
+        <v>162991</v>
       </c>
       <c r="J288" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K288" s="2" t="inlineStr">
         <is>
@@ -28176,10 +28176,10 @@
         <v>11612</v>
       </c>
       <c r="I289" s="2" t="n">
-        <v>100840</v>
+        <v>112452</v>
       </c>
       <c r="J289" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K289" s="2" t="inlineStr">
         <is>
@@ -28368,10 +28368,10 @@
         <v>11499</v>
       </c>
       <c r="I291" s="2" t="n">
-        <v>78555</v>
+        <v>90054</v>
       </c>
       <c r="J291" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K291" s="2" t="inlineStr">
         <is>
@@ -28752,10 +28752,10 @@
         <v>11226</v>
       </c>
       <c r="I295" s="2" t="n">
-        <v>103246</v>
+        <v>110078</v>
       </c>
       <c r="J295" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K295" s="2" t="inlineStr">
         <is>
@@ -28848,10 +28848,10 @@
         <v>10989</v>
       </c>
       <c r="I296" s="2" t="n">
-        <v>109189</v>
+        <v>111114</v>
       </c>
       <c r="J296" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K296" s="2" t="inlineStr">
         <is>
@@ -28944,10 +28944,10 @@
         <v>10726</v>
       </c>
       <c r="I297" s="2" t="n">
-        <v>152128</v>
+        <v>154664</v>
       </c>
       <c r="J297" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K297" s="2" t="inlineStr">
         <is>
@@ -29040,10 +29040,10 @@
         <v>10675</v>
       </c>
       <c r="I298" s="2" t="n">
-        <v>66982</v>
+        <v>74164</v>
       </c>
       <c r="J298" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K298" s="2" t="inlineStr">
         <is>
@@ -29232,10 +29232,10 @@
         <v>10641</v>
       </c>
       <c r="I300" s="2" t="n">
-        <v>63428</v>
+        <v>68644</v>
       </c>
       <c r="J300" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K300" s="2" t="inlineStr">
         <is>
@@ -29328,10 +29328,10 @@
         <v>10325</v>
       </c>
       <c r="I301" s="2" t="n">
-        <v>50406</v>
+        <v>53951</v>
       </c>
       <c r="J301" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K301" s="2" t="inlineStr">
         <is>
@@ -29424,10 +29424,10 @@
         <v>10316</v>
       </c>
       <c r="I302" s="2" t="n">
-        <v>94566</v>
+        <v>96020</v>
       </c>
       <c r="J302" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K302" s="2" t="inlineStr">
         <is>
@@ -29520,10 +29520,10 @@
         <v>10306</v>
       </c>
       <c r="I303" s="2" t="n">
-        <v>86407</v>
+        <v>89561</v>
       </c>
       <c r="J303" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K303" s="2" t="inlineStr">
         <is>
@@ -29616,10 +29616,10 @@
         <v>10268</v>
       </c>
       <c r="I304" s="2" t="n">
-        <v>114465</v>
+        <v>116935</v>
       </c>
       <c r="J304" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K304" s="2" t="inlineStr">
         <is>
@@ -29712,10 +29712,10 @@
         <v>10190</v>
       </c>
       <c r="I305" s="2" t="n">
-        <v>123738</v>
+        <v>130046</v>
       </c>
       <c r="J305" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K305" s="2" t="inlineStr">
         <is>
@@ -29808,10 +29808,10 @@
         <v>10127</v>
       </c>
       <c r="I306" s="2" t="n">
-        <v>42505</v>
+        <v>44432</v>
       </c>
       <c r="J306" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K306" s="2" t="inlineStr">
         <is>
@@ -30096,10 +30096,10 @@
         <v>10057</v>
       </c>
       <c r="I309" s="2" t="n">
-        <v>151104</v>
+        <v>160282</v>
       </c>
       <c r="J309" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K309" s="2" t="inlineStr">
         <is>
@@ -30192,10 +30192,10 @@
         <v>10043</v>
       </c>
       <c r="I310" s="2" t="n">
-        <v>80836</v>
+        <v>90879</v>
       </c>
       <c r="J310" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K310" s="2" t="inlineStr">
         <is>
@@ -30768,10 +30768,10 @@
         <v>9863</v>
       </c>
       <c r="I316" s="2" t="n">
-        <v>126104</v>
+        <v>130331</v>
       </c>
       <c r="J316" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K316" s="2" t="inlineStr">
         <is>
@@ -30864,10 +30864,10 @@
         <v>9823</v>
       </c>
       <c r="I317" s="2" t="n">
-        <v>84130</v>
+        <v>87077</v>
       </c>
       <c r="J317" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K317" s="2" t="inlineStr">
         <is>
@@ -30960,10 +30960,10 @@
         <v>9814</v>
       </c>
       <c r="I318" s="2" t="n">
-        <v>106275</v>
+        <v>108227</v>
       </c>
       <c r="J318" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K318" s="2" t="inlineStr">
         <is>
@@ -31152,10 +31152,10 @@
         <v>9795</v>
       </c>
       <c r="I320" s="2" t="n">
-        <v>98256</v>
+        <v>106488</v>
       </c>
       <c r="J320" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K320" s="2" t="inlineStr">
         <is>
@@ -31248,10 +31248,10 @@
         <v>9763</v>
       </c>
       <c r="I321" s="2" t="n">
-        <v>48814</v>
+        <v>53695</v>
       </c>
       <c r="J321" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
@@ -31728,10 +31728,10 @@
         <v>9631</v>
       </c>
       <c r="I326" s="2" t="n">
-        <v>66464</v>
+        <v>69355</v>
       </c>
       <c r="J326" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K326" s="2" t="inlineStr">
         <is>
@@ -31824,10 +31824,10 @@
         <v>9608</v>
       </c>
       <c r="I327" s="2" t="n">
-        <v>30376</v>
+        <v>31726</v>
       </c>
       <c r="J327" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K327" s="2" t="inlineStr">
         <is>
@@ -31920,10 +31920,10 @@
         <v>9587</v>
       </c>
       <c r="I328" s="2" t="n">
-        <v>114685</v>
+        <v>118376</v>
       </c>
       <c r="J328" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K328" s="2" t="inlineStr">
         <is>
@@ -32304,10 +32304,10 @@
         <v>9503</v>
       </c>
       <c r="I332" s="2" t="n">
-        <v>125835</v>
+        <v>129257</v>
       </c>
       <c r="J332" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K332" s="2" t="inlineStr">
         <is>
@@ -32400,10 +32400,10 @@
         <v>9470</v>
       </c>
       <c r="I333" s="2" t="n">
-        <v>173119</v>
+        <v>182370</v>
       </c>
       <c r="J333" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K333" s="2" t="inlineStr">
         <is>
@@ -32496,10 +32496,10 @@
         <v>9348</v>
       </c>
       <c r="I334" s="2" t="n">
-        <v>116732</v>
+        <v>118660</v>
       </c>
       <c r="J334" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K334" s="2" t="inlineStr">
         <is>
@@ -32592,10 +32592,10 @@
         <v>9306</v>
       </c>
       <c r="I335" s="2" t="n">
-        <v>126951</v>
+        <v>132027</v>
       </c>
       <c r="J335" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K335" s="2" t="inlineStr">
         <is>
@@ -32688,10 +32688,10 @@
         <v>9274</v>
       </c>
       <c r="I336" s="2" t="n">
-        <v>123416</v>
+        <v>126832</v>
       </c>
       <c r="J336" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K336" s="2" t="inlineStr">
         <is>
@@ -32784,10 +32784,10 @@
         <v>9236</v>
       </c>
       <c r="I337" s="2" t="n">
-        <v>46531</v>
+        <v>51449</v>
       </c>
       <c r="J337" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K337" s="2" t="inlineStr">
         <is>
@@ -32880,10 +32880,10 @@
         <v>9152</v>
       </c>
       <c r="I338" s="2" t="n">
-        <v>100344</v>
+        <v>102218</v>
       </c>
       <c r="J338" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
@@ -33168,10 +33168,10 @@
         <v>9047</v>
       </c>
       <c r="I341" s="2" t="n">
-        <v>97197</v>
+        <v>101720</v>
       </c>
       <c r="J341" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K341" s="2" t="inlineStr">
         <is>
@@ -33264,10 +33264,10 @@
         <v>9028</v>
       </c>
       <c r="I342" s="2" t="n">
-        <v>56930</v>
+        <v>65129</v>
       </c>
       <c r="J342" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
@@ -33456,10 +33456,10 @@
         <v>8982</v>
       </c>
       <c r="I344" s="2" t="n">
-        <v>133591</v>
+        <v>142573</v>
       </c>
       <c r="J344" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K344" s="2" t="inlineStr">
         <is>
@@ -33840,10 +33840,10 @@
         <v>8847</v>
       </c>
       <c r="I348" s="2" t="n">
-        <v>163469</v>
+        <v>171190</v>
       </c>
       <c r="J348" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K348" s="2" t="inlineStr">
         <is>
@@ -34320,10 +34320,10 @@
         <v>8739</v>
       </c>
       <c r="I353" s="2" t="n">
-        <v>69908</v>
+        <v>78647</v>
       </c>
       <c r="J353" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K353" s="2" t="inlineStr">
         <is>
@@ -34416,10 +34416,10 @@
         <v>8726</v>
       </c>
       <c r="I354" s="2" t="n">
-        <v>155372</v>
+        <v>157809</v>
       </c>
       <c r="J354" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K354" s="2" t="inlineStr">
         <is>
@@ -34608,10 +34608,10 @@
         <v>8653</v>
       </c>
       <c r="I356" s="2" t="n">
-        <v>126042</v>
+        <v>130933</v>
       </c>
       <c r="J356" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
@@ -34800,10 +34800,10 @@
         <v>8643</v>
       </c>
       <c r="I358" s="2" t="n">
-        <v>56503</v>
+        <v>63255</v>
       </c>
       <c r="J358" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K358" s="2" t="inlineStr">
         <is>
@@ -34896,10 +34896,10 @@
         <v>8585</v>
       </c>
       <c r="I359" s="2" t="n">
-        <v>94643</v>
+        <v>100349</v>
       </c>
       <c r="J359" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
@@ -35088,10 +35088,10 @@
         <v>8467</v>
       </c>
       <c r="I361" s="2" t="n">
-        <v>79961</v>
+        <v>86076</v>
       </c>
       <c r="J361" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K361" s="2" t="inlineStr">
         <is>
@@ -35184,10 +35184,10 @@
         <v>8464</v>
       </c>
       <c r="I362" s="2" t="n">
-        <v>67708</v>
+        <v>76172</v>
       </c>
       <c r="J362" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K362" s="2" t="inlineStr">
         <is>
@@ -35376,10 +35376,10 @@
         <v>8341</v>
       </c>
       <c r="I364" s="2" t="n">
-        <v>93572</v>
+        <v>101913</v>
       </c>
       <c r="J364" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K364" s="2" t="inlineStr">
         <is>
@@ -35856,10 +35856,10 @@
         <v>8136</v>
       </c>
       <c r="I369" s="2" t="n">
-        <v>64664</v>
+        <v>70599</v>
       </c>
       <c r="J369" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K369" s="2" t="inlineStr">
         <is>
@@ -36048,10 +36048,10 @@
         <v>8100</v>
       </c>
       <c r="I371" s="2" t="n">
-        <v>16200</v>
+        <v>24300</v>
       </c>
       <c r="J371" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K371" s="2" t="inlineStr">
         <is>
@@ -36240,10 +36240,10 @@
         <v>8084</v>
       </c>
       <c r="I373" s="2" t="n">
-        <v>44003</v>
+        <v>45440</v>
       </c>
       <c r="J373" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K373" s="2" t="inlineStr">
         <is>
@@ -36432,10 +36432,10 @@
         <v>7997</v>
       </c>
       <c r="I375" s="2" t="n">
-        <v>76574</v>
+        <v>82784</v>
       </c>
       <c r="J375" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K375" s="2" t="inlineStr">
         <is>
@@ -36528,10 +36528,10 @@
         <v>7825</v>
       </c>
       <c r="I376" s="2" t="n">
-        <v>100696</v>
+        <v>108521</v>
       </c>
       <c r="J376" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K376" s="2" t="inlineStr">
         <is>
@@ -36624,10 +36624,10 @@
         <v>7811</v>
       </c>
       <c r="I377" s="2" t="n">
-        <v>64398</v>
+        <v>70686</v>
       </c>
       <c r="J377" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K377" s="2" t="inlineStr">
         <is>
@@ -37392,10 +37392,10 @@
         <v>7524</v>
       </c>
       <c r="I385" s="2" t="n">
-        <v>50787</v>
+        <v>54549</v>
       </c>
       <c r="J385" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K385" s="2" t="inlineStr">
         <is>
@@ -37680,10 +37680,10 @@
         <v>7477</v>
       </c>
       <c r="I388" s="2" t="n">
-        <v>45820</v>
+        <v>52531</v>
       </c>
       <c r="J388" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K388" s="2" t="inlineStr">
         <is>
@@ -37776,10 +37776,10 @@
         <v>7428</v>
       </c>
       <c r="I389" s="2" t="n">
-        <v>52384</v>
+        <v>54003</v>
       </c>
       <c r="J389" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K389" s="2" t="inlineStr">
         <is>
@@ -37872,10 +37872,10 @@
         <v>7420</v>
       </c>
       <c r="I390" s="2" t="n">
-        <v>90307</v>
+        <v>95545</v>
       </c>
       <c r="J390" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K390" s="2" t="inlineStr">
         <is>
@@ -37968,10 +37968,10 @@
         <v>7233</v>
       </c>
       <c r="I391" s="2" t="n">
-        <v>69915</v>
+        <v>77148</v>
       </c>
       <c r="J391" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K391" s="2" t="inlineStr">
         <is>
@@ -38064,10 +38064,10 @@
         <v>7197</v>
       </c>
       <c r="I392" s="2" t="n">
-        <v>75072</v>
+        <v>77290</v>
       </c>
       <c r="J392" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K392" s="2" t="inlineStr">
         <is>
@@ -38160,10 +38160,10 @@
         <v>7172</v>
       </c>
       <c r="I393" s="2" t="n">
-        <v>50110</v>
+        <v>54860</v>
       </c>
       <c r="J393" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K393" s="2" t="inlineStr">
         <is>
@@ -38256,10 +38256,10 @@
         <v>7135</v>
       </c>
       <c r="I394" s="2" t="n">
-        <v>73224</v>
+        <v>79701</v>
       </c>
       <c r="J394" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K394" s="2" t="inlineStr">
         <is>
@@ -38448,10 +38448,10 @@
         <v>7073</v>
       </c>
       <c r="I396" s="2" t="n">
-        <v>42140</v>
+        <v>49064</v>
       </c>
       <c r="J396" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K396" s="2" t="inlineStr">
         <is>
@@ -38544,10 +38544,10 @@
         <v>7017</v>
       </c>
       <c r="I397" s="2" t="n">
-        <v>54756</v>
+        <v>61773</v>
       </c>
       <c r="J397" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K397" s="2" t="inlineStr">
         <is>
@@ -38736,10 +38736,10 @@
         <v>6924</v>
       </c>
       <c r="I399" s="2" t="n">
-        <v>27687</v>
+        <v>34611</v>
       </c>
       <c r="J399" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K399" s="2" t="inlineStr">
         <is>
@@ -38928,10 +38928,10 @@
         <v>6873</v>
       </c>
       <c r="I401" s="2" t="n">
-        <v>64814</v>
+        <v>71687</v>
       </c>
       <c r="J401" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K401" s="2" t="inlineStr">
         <is>
@@ -39120,10 +39120,10 @@
         <v>6833</v>
       </c>
       <c r="I403" s="2" t="n">
-        <v>31234</v>
+        <v>34162</v>
       </c>
       <c r="J403" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K403" s="2" t="inlineStr">
         <is>
@@ -39408,10 +39408,10 @@
         <v>6681</v>
       </c>
       <c r="I406" s="2" t="n">
-        <v>15244</v>
+        <v>21925</v>
       </c>
       <c r="J406" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K406" s="2" t="inlineStr">
         <is>
@@ -39504,10 +39504,10 @@
         <v>6666</v>
       </c>
       <c r="I407" s="2" t="n">
-        <v>56186</v>
+        <v>59519</v>
       </c>
       <c r="J407" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K407" s="2" t="inlineStr">
         <is>
@@ -39696,10 +39696,10 @@
         <v>6588</v>
       </c>
       <c r="I409" s="2" t="n">
-        <v>26348</v>
+        <v>32934</v>
       </c>
       <c r="J409" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K409" s="2" t="inlineStr">
         <is>
@@ -39792,10 +39792,10 @@
         <v>6585</v>
       </c>
       <c r="I410" s="2" t="n">
-        <v>95012</v>
+        <v>98305</v>
       </c>
       <c r="J410" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K410" s="2" t="inlineStr">
         <is>
@@ -39984,10 +39984,10 @@
         <v>6584</v>
       </c>
       <c r="I412" s="2" t="n">
-        <v>50788</v>
+        <v>57372</v>
       </c>
       <c r="J412" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K412" s="2" t="inlineStr">
         <is>
@@ -40080,10 +40080,10 @@
         <v>6578</v>
       </c>
       <c r="I413" s="2" t="n">
-        <v>61148</v>
+        <v>64633</v>
       </c>
       <c r="J413" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K413" s="2" t="inlineStr">
         <is>
@@ -40272,10 +40272,10 @@
         <v>6554</v>
       </c>
       <c r="I415" s="2" t="n">
-        <v>19226</v>
+        <v>20634</v>
       </c>
       <c r="J415" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K415" s="2" t="inlineStr">
         <is>
@@ -40368,10 +40368,10 @@
         <v>6548</v>
       </c>
       <c r="I416" s="2" t="n">
-        <v>13096</v>
+        <v>19644</v>
       </c>
       <c r="J416" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K416" s="2" t="inlineStr">
         <is>
@@ -40464,10 +40464,10 @@
         <v>6529</v>
       </c>
       <c r="I417" s="2" t="n">
-        <v>51310</v>
+        <v>57839</v>
       </c>
       <c r="J417" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K417" s="2" t="inlineStr">
         <is>
@@ -40560,10 +40560,10 @@
         <v>6522</v>
       </c>
       <c r="I418" s="2" t="n">
-        <v>104162</v>
+        <v>107917</v>
       </c>
       <c r="J418" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K418" s="2" t="inlineStr">
         <is>
@@ -40944,10 +40944,10 @@
         <v>6402</v>
       </c>
       <c r="I422" s="2" t="n">
-        <v>21284</v>
+        <v>23404</v>
       </c>
       <c r="J422" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K422" s="2" t="inlineStr">
         <is>
@@ -41136,10 +41136,10 @@
         <v>6365</v>
       </c>
       <c r="I424" s="2" t="n">
-        <v>26534</v>
+        <v>28506</v>
       </c>
       <c r="J424" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K424" s="2" t="inlineStr">
         <is>
@@ -41328,10 +41328,10 @@
         <v>6286</v>
       </c>
       <c r="I426" s="2" t="n">
-        <v>57050</v>
+        <v>61414</v>
       </c>
       <c r="J426" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K426" s="2" t="inlineStr">
         <is>
@@ -41712,10 +41712,10 @@
         <v>6232</v>
       </c>
       <c r="I430" s="2" t="n">
-        <v>77308</v>
+        <v>81188</v>
       </c>
       <c r="J430" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K430" s="2" t="inlineStr">
         <is>
@@ -41904,10 +41904,10 @@
         <v>6190</v>
       </c>
       <c r="I432" s="2" t="n">
-        <v>12380</v>
+        <v>18570</v>
       </c>
       <c r="J432" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K432" s="2" t="inlineStr">
         <is>
@@ -42000,10 +42000,10 @@
         <v>6117</v>
       </c>
       <c r="I433" s="2" t="n">
-        <v>71664</v>
+        <v>72830</v>
       </c>
       <c r="J433" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K433" s="2" t="inlineStr">
         <is>
@@ -42096,10 +42096,10 @@
         <v>6115</v>
       </c>
       <c r="I434" s="2" t="n">
-        <v>42333</v>
+        <v>48448</v>
       </c>
       <c r="J434" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K434" s="2" t="inlineStr">
         <is>
@@ -42288,10 +42288,10 @@
         <v>6047</v>
       </c>
       <c r="I436" s="2" t="n">
-        <v>50351</v>
+        <v>54988</v>
       </c>
       <c r="J436" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K436" s="2" t="inlineStr">
         <is>
@@ -42384,10 +42384,10 @@
         <v>5956</v>
       </c>
       <c r="I437" s="2" t="n">
-        <v>46085</v>
+        <v>48526</v>
       </c>
       <c r="J437" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K437" s="2" t="inlineStr">
         <is>
@@ -42480,10 +42480,10 @@
         <v>5927</v>
       </c>
       <c r="I438" s="2" t="n">
-        <v>74090</v>
+        <v>79030</v>
       </c>
       <c r="J438" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K438" s="2" t="inlineStr">
         <is>
@@ -42576,10 +42576,10 @@
         <v>5912</v>
       </c>
       <c r="I439" s="2" t="n">
-        <v>45052</v>
+        <v>48993</v>
       </c>
       <c r="J439" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K439" s="2" t="inlineStr">
         <is>
@@ -42672,10 +42672,10 @@
         <v>5858</v>
       </c>
       <c r="I440" s="2" t="n">
-        <v>38024</v>
+        <v>40953</v>
       </c>
       <c r="J440" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K440" s="2" t="inlineStr">
         <is>
@@ -42864,10 +42864,10 @@
         <v>5857</v>
       </c>
       <c r="I442" s="2" t="n">
-        <v>11714</v>
+        <v>17571</v>
       </c>
       <c r="J442" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K442" s="2" t="inlineStr">
         <is>
@@ -43056,10 +43056,10 @@
         <v>5846</v>
       </c>
       <c r="I444" s="2" t="n">
-        <v>68906</v>
+        <v>70490</v>
       </c>
       <c r="J444" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K444" s="2" t="inlineStr">
         <is>
@@ -43248,10 +43248,10 @@
         <v>5834</v>
       </c>
       <c r="I446" s="2" t="n">
-        <v>68690</v>
+        <v>71231</v>
       </c>
       <c r="J446" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K446" s="2" t="inlineStr">
         <is>
@@ -43728,10 +43728,10 @@
         <v>5674</v>
       </c>
       <c r="I451" s="2" t="n">
-        <v>84792</v>
+        <v>88924</v>
       </c>
       <c r="J451" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K451" s="2" t="inlineStr">
         <is>
@@ -43920,10 +43920,10 @@
         <v>5644</v>
       </c>
       <c r="I453" s="2" t="n">
-        <v>31042</v>
+        <v>36686</v>
       </c>
       <c r="J453" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K453" s="2" t="inlineStr">
         <is>
@@ -44016,10 +44016,10 @@
         <v>5643</v>
       </c>
       <c r="I454" s="2" t="n">
-        <v>89413</v>
+        <v>92235</v>
       </c>
       <c r="J454" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K454" s="2" t="inlineStr">
         <is>
@@ -44496,10 +44496,10 @@
         <v>5496</v>
       </c>
       <c r="I459" s="2" t="n">
-        <v>36831</v>
+        <v>40206</v>
       </c>
       <c r="J459" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K459" s="2" t="inlineStr">
         <is>
@@ -44592,10 +44592,10 @@
         <v>5468</v>
       </c>
       <c r="I460" s="2" t="n">
-        <v>36314</v>
+        <v>41782</v>
       </c>
       <c r="J460" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K460" s="2" t="inlineStr">
         <is>
@@ -44688,10 +44688,10 @@
         <v>5420</v>
       </c>
       <c r="I461" s="2" t="n">
-        <v>77847</v>
+        <v>79881</v>
       </c>
       <c r="J461" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K461" s="2" t="inlineStr">
         <is>
@@ -44880,10 +44880,10 @@
         <v>5400</v>
       </c>
       <c r="I463" s="2" t="n">
-        <v>48372</v>
+        <v>52324</v>
       </c>
       <c r="J463" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K463" s="2" t="inlineStr">
         <is>
@@ -45072,10 +45072,10 @@
         <v>5399</v>
       </c>
       <c r="I465" s="2" t="n">
-        <v>16196</v>
+        <v>21595</v>
       </c>
       <c r="J465" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K465" s="2" t="inlineStr">
         <is>
@@ -45552,10 +45552,10 @@
         <v>5356</v>
       </c>
       <c r="I470" s="2" t="n">
-        <v>70403</v>
+        <v>75759</v>
       </c>
       <c r="J470" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K470" s="2" t="inlineStr">
         <is>
@@ -45744,10 +45744,10 @@
         <v>5268</v>
       </c>
       <c r="I472" s="2" t="n">
-        <v>48354</v>
+        <v>50706</v>
       </c>
       <c r="J472" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K472" s="2" t="inlineStr">
         <is>
@@ -45840,10 +45840,10 @@
         <v>5267</v>
       </c>
       <c r="I473" s="2" t="n">
-        <v>24454</v>
+        <v>29721</v>
       </c>
       <c r="J473" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K473" s="2" t="inlineStr">
         <is>
@@ -45936,10 +45936,10 @@
         <v>5263</v>
       </c>
       <c r="I474" s="2" t="n">
-        <v>10526</v>
+        <v>15789</v>
       </c>
       <c r="J474" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K474" s="2" t="inlineStr">
         <is>
@@ -46416,10 +46416,10 @@
         <v>5176</v>
       </c>
       <c r="I479" s="2" t="n">
-        <v>79051</v>
+        <v>80463</v>
       </c>
       <c r="J479" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K479" s="2" t="inlineStr">
         <is>
@@ -46512,10 +46512,10 @@
         <v>5174</v>
       </c>
       <c r="I480" s="2" t="n">
-        <v>61334</v>
+        <v>62933</v>
       </c>
       <c r="J480" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K480" s="2" t="inlineStr">
         <is>
@@ -46992,10 +46992,10 @@
         <v>5027</v>
       </c>
       <c r="I485" s="2" t="n">
-        <v>61101</v>
+        <v>62362</v>
       </c>
       <c r="J485" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K485" s="2" t="inlineStr">
         <is>
@@ -47088,10 +47088,10 @@
         <v>5004</v>
       </c>
       <c r="I486" s="2" t="n">
-        <v>31017</v>
+        <v>33013</v>
       </c>
       <c r="J486" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K486" s="2" t="inlineStr">
         <is>
@@ -47472,10 +47472,10 @@
         <v>4880</v>
       </c>
       <c r="I490" s="2" t="n">
-        <v>29670</v>
+        <v>32598</v>
       </c>
       <c r="J490" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K490" s="2" t="inlineStr">
         <is>
@@ -47664,10 +47664,10 @@
         <v>4860</v>
       </c>
       <c r="I492" s="2" t="n">
-        <v>28620</v>
+        <v>33480</v>
       </c>
       <c r="J492" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K492" s="2" t="inlineStr">
         <is>
@@ -47952,10 +47952,10 @@
         <v>4851</v>
       </c>
       <c r="I495" s="2" t="n">
-        <v>44141</v>
+        <v>47052</v>
       </c>
       <c r="J495" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K495" s="2" t="inlineStr">
         <is>
@@ -48144,10 +48144,10 @@
         <v>4840</v>
       </c>
       <c r="I497" s="2" t="n">
-        <v>70301</v>
+        <v>75141</v>
       </c>
       <c r="J497" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K497" s="2" t="inlineStr">
         <is>
@@ -48528,10 +48528,10 @@
         <v>4813</v>
       </c>
       <c r="I501" s="2" t="n">
-        <v>62360</v>
+        <v>67173</v>
       </c>
       <c r="J501" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K501" s="2" t="inlineStr">
         <is>
@@ -48624,10 +48624,10 @@
         <v>4798</v>
       </c>
       <c r="I502" s="2" t="n">
-        <v>36584</v>
+        <v>38083</v>
       </c>
       <c r="J502" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K502" s="2" t="inlineStr">
         <is>
@@ -48912,10 +48912,10 @@
         <v>4705</v>
       </c>
       <c r="I505" s="2" t="n">
-        <v>51756</v>
+        <v>54109</v>
       </c>
       <c r="J505" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K505" s="2" t="inlineStr">
         <is>
@@ -49296,10 +49296,10 @@
         <v>4552</v>
       </c>
       <c r="I509" s="2" t="n">
-        <v>9104</v>
+        <v>13656</v>
       </c>
       <c r="J509" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K509" s="2" t="inlineStr">
         <is>
@@ -50064,10 +50064,10 @@
         <v>4288</v>
       </c>
       <c r="I517" s="2" t="n">
-        <v>8576</v>
+        <v>12864</v>
       </c>
       <c r="J517" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K517" s="2" t="inlineStr">
         <is>
@@ -50256,10 +50256,10 @@
         <v>4216</v>
       </c>
       <c r="I519" s="2" t="n">
-        <v>8432</v>
+        <v>12648</v>
       </c>
       <c r="J519" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K519" s="2" t="inlineStr">
         <is>
@@ -50448,10 +50448,10 @@
         <v>4002</v>
       </c>
       <c r="I521" s="2" t="n">
-        <v>31347</v>
+        <v>35349</v>
       </c>
       <c r="J521" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K521" s="2" t="inlineStr">
         <is>
@@ -50544,10 +50544,10 @@
         <v>3975</v>
       </c>
       <c r="I522" s="2" t="n">
-        <v>46708</v>
+        <v>50683</v>
       </c>
       <c r="J522" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K522" s="2" t="inlineStr">
         <is>
@@ -50640,10 +50640,10 @@
         <v>3960</v>
       </c>
       <c r="I523" s="2" t="n">
-        <v>14040</v>
+        <v>18000</v>
       </c>
       <c r="J523" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K523" s="2" t="inlineStr">
         <is>
@@ -50736,10 +50736,10 @@
         <v>3952</v>
       </c>
       <c r="I524" s="2" t="n">
-        <v>50584</v>
+        <v>52560</v>
       </c>
       <c r="J524" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K524" s="2" t="inlineStr">
         <is>
@@ -51024,10 +51024,10 @@
         <v>3942</v>
       </c>
       <c r="I527" s="2" t="n">
-        <v>79931</v>
+        <v>83652</v>
       </c>
       <c r="J527" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K527" s="2" t="inlineStr">
         <is>
@@ -51120,10 +51120,10 @@
         <v>3942</v>
       </c>
       <c r="I528" s="2" t="n">
-        <v>7884</v>
+        <v>11826</v>
       </c>
       <c r="J528" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K528" s="2" t="inlineStr">
         <is>
@@ -51216,10 +51216,10 @@
         <v>3941</v>
       </c>
       <c r="I529" s="2" t="n">
-        <v>11824</v>
+        <v>13795</v>
       </c>
       <c r="J529" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K529" s="2" t="inlineStr">
         <is>
@@ -51408,10 +51408,10 @@
         <v>3927</v>
       </c>
       <c r="I531" s="2" t="n">
-        <v>76049</v>
+        <v>78013</v>
       </c>
       <c r="J531" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K531" s="2" t="inlineStr">
         <is>
@@ -51504,10 +51504,10 @@
         <v>3925</v>
       </c>
       <c r="I532" s="2" t="n">
-        <v>19628</v>
+        <v>21591</v>
       </c>
       <c r="J532" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K532" s="2" t="inlineStr">
         <is>
@@ -51600,10 +51600,10 @@
         <v>3905</v>
       </c>
       <c r="I533" s="2" t="n">
-        <v>21476</v>
+        <v>24404</v>
       </c>
       <c r="J533" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K533" s="2" t="inlineStr">
         <is>
@@ -51792,10 +51792,10 @@
         <v>3878</v>
       </c>
       <c r="I535" s="2" t="n">
-        <v>56231</v>
+        <v>58170</v>
       </c>
       <c r="J535" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K535" s="2" t="inlineStr">
         <is>
@@ -52080,10 +52080,10 @@
         <v>3856</v>
       </c>
       <c r="I538" s="2" t="n">
-        <v>36632</v>
+        <v>40488</v>
       </c>
       <c r="J538" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K538" s="2" t="inlineStr">
         <is>
@@ -52176,10 +52176,10 @@
         <v>3835</v>
       </c>
       <c r="I539" s="2" t="n">
-        <v>7670</v>
+        <v>11505</v>
       </c>
       <c r="J539" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K539" s="2" t="inlineStr">
         <is>
@@ -52752,10 +52752,10 @@
         <v>3764</v>
       </c>
       <c r="I545" s="2" t="n">
-        <v>61729</v>
+        <v>63235</v>
       </c>
       <c r="J545" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K545" s="2" t="inlineStr">
         <is>
@@ -53136,10 +53136,10 @@
         <v>3763</v>
       </c>
       <c r="I549" s="2" t="n">
-        <v>7526</v>
+        <v>11289</v>
       </c>
       <c r="J549" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K549" s="2" t="inlineStr">
         <is>
@@ -53232,10 +53232,10 @@
         <v>3762</v>
       </c>
       <c r="I550" s="2" t="n">
-        <v>40047</v>
+        <v>41738</v>
       </c>
       <c r="J550" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K550" s="2" t="inlineStr">
         <is>
@@ -53328,10 +53328,10 @@
         <v>3755</v>
       </c>
       <c r="I551" s="2" t="n">
-        <v>61526</v>
+        <v>63874</v>
       </c>
       <c r="J551" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K551" s="2" t="inlineStr">
         <is>
@@ -53424,10 +53424,10 @@
         <v>3736</v>
       </c>
       <c r="I552" s="2" t="n">
-        <v>50721</v>
+        <v>52637</v>
       </c>
       <c r="J552" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K552" s="2" t="inlineStr">
         <is>
@@ -53616,10 +53616,10 @@
         <v>3732</v>
       </c>
       <c r="I554" s="2" t="n">
-        <v>45764</v>
+        <v>47728</v>
       </c>
       <c r="J554" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K554" s="2" t="inlineStr">
         <is>
@@ -53808,10 +53808,10 @@
         <v>3675</v>
       </c>
       <c r="I556" s="2" t="n">
-        <v>20328</v>
+        <v>24003</v>
       </c>
       <c r="J556" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K556" s="2" t="inlineStr">
         <is>
@@ -53904,10 +53904,10 @@
         <v>3600</v>
       </c>
       <c r="I557" s="2" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="J557" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K557" s="2" t="inlineStr">
         <is>
@@ -54000,10 +54000,10 @@
         <v>3597</v>
       </c>
       <c r="I558" s="2" t="n">
-        <v>14389</v>
+        <v>17986</v>
       </c>
       <c r="J558" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K558" s="2" t="inlineStr">
         <is>
@@ -54384,10 +54384,10 @@
         <v>3469</v>
       </c>
       <c r="I562" s="2" t="n">
-        <v>29998</v>
+        <v>32123</v>
       </c>
       <c r="J562" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K562" s="2" t="inlineStr">
         <is>
@@ -54480,10 +54480,10 @@
         <v>3428</v>
       </c>
       <c r="I563" s="2" t="n">
-        <v>31992</v>
+        <v>35420</v>
       </c>
       <c r="J563" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K563" s="2" t="inlineStr">
         <is>
@@ -54768,10 +54768,10 @@
         <v>3407</v>
       </c>
       <c r="I566" s="2" t="n">
-        <v>19982</v>
+        <v>23389</v>
       </c>
       <c r="J566" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K566" s="2" t="inlineStr">
         <is>
@@ -55056,10 +55056,10 @@
         <v>3375</v>
       </c>
       <c r="I569" s="2" t="n">
-        <v>33750</v>
+        <v>37125</v>
       </c>
       <c r="J569" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K569" s="2" t="inlineStr">
         <is>
@@ -55440,10 +55440,10 @@
         <v>3327</v>
       </c>
       <c r="I573" s="2" t="n">
-        <v>6654</v>
+        <v>9981</v>
       </c>
       <c r="J573" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K573" s="2" t="inlineStr">
         <is>
@@ -55920,10 +55920,10 @@
         <v>3292</v>
       </c>
       <c r="I578" s="2" t="n">
-        <v>6584</v>
+        <v>9876</v>
       </c>
       <c r="J578" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K578" s="2" t="inlineStr">
         <is>
@@ -56016,10 +56016,10 @@
         <v>3232</v>
       </c>
       <c r="I579" s="2" t="n">
-        <v>16160</v>
+        <v>17776</v>
       </c>
       <c r="J579" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K579" s="2" t="inlineStr">
         <is>
@@ -56112,10 +56112,10 @@
         <v>3210</v>
       </c>
       <c r="I580" s="2" t="n">
-        <v>6420</v>
+        <v>9630</v>
       </c>
       <c r="J580" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K580" s="2" t="inlineStr">
         <is>
@@ -56208,10 +56208,10 @@
         <v>3144</v>
       </c>
       <c r="I581" s="2" t="n">
-        <v>28776</v>
+        <v>30872</v>
       </c>
       <c r="J581" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K581" s="2" t="inlineStr">
         <is>
@@ -56304,10 +56304,10 @@
         <v>3103</v>
       </c>
       <c r="I582" s="2" t="n">
-        <v>28394</v>
+        <v>30275</v>
       </c>
       <c r="J582" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K582" s="2" t="inlineStr">
         <is>
@@ -56400,10 +56400,10 @@
         <v>3066</v>
       </c>
       <c r="I583" s="2" t="n">
-        <v>9964</v>
+        <v>13030</v>
       </c>
       <c r="J583" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K583" s="2" t="inlineStr">
         <is>
@@ -56496,10 +56496,10 @@
         <v>3060</v>
       </c>
       <c r="I584" s="2" t="n">
-        <v>25920</v>
+        <v>28440</v>
       </c>
       <c r="J584" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
@@ -56688,10 +56688,10 @@
         <v>3007</v>
       </c>
       <c r="I586" s="2" t="n">
-        <v>6014</v>
+        <v>9021</v>
       </c>
       <c r="J586" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
@@ -56880,10 +56880,10 @@
         <v>2953</v>
       </c>
       <c r="I588" s="2" t="n">
-        <v>5906</v>
+        <v>8859</v>
       </c>
       <c r="J588" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
@@ -57456,10 +57456,10 @@
         <v>2911</v>
       </c>
       <c r="I594" s="2" t="n">
-        <v>33959</v>
+        <v>35899</v>
       </c>
       <c r="J594" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
@@ -57552,10 +57552,10 @@
         <v>2909</v>
       </c>
       <c r="I595" s="2" t="n">
-        <v>21890</v>
+        <v>23359</v>
       </c>
       <c r="J595" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K595" s="2" t="inlineStr">
         <is>
@@ -57744,10 +57744,10 @@
         <v>2898</v>
       </c>
       <c r="I597" s="2" t="n">
-        <v>28311</v>
+        <v>29522</v>
       </c>
       <c r="J597" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K597" s="2" t="inlineStr">
         <is>
@@ -58512,10 +58512,10 @@
         <v>2863</v>
       </c>
       <c r="I605" s="2" t="n">
-        <v>46526</v>
+        <v>48778</v>
       </c>
       <c r="J605" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K605" s="2" t="inlineStr">
         <is>
@@ -58800,10 +58800,10 @@
         <v>2850</v>
       </c>
       <c r="I608" s="2" t="n">
-        <v>5700</v>
+        <v>8550</v>
       </c>
       <c r="J608" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
@@ -58896,10 +58896,10 @@
         <v>2826</v>
       </c>
       <c r="I609" s="2" t="n">
-        <v>11186</v>
+        <v>13953</v>
       </c>
       <c r="J609" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K609" s="2" t="inlineStr">
         <is>
@@ -59376,10 +59376,10 @@
         <v>2822</v>
       </c>
       <c r="I614" s="2" t="n">
-        <v>24458</v>
+        <v>26810</v>
       </c>
       <c r="J614" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K614" s="2" t="inlineStr">
         <is>
@@ -59472,10 +59472,10 @@
         <v>2822</v>
       </c>
       <c r="I615" s="2" t="n">
-        <v>30099</v>
+        <v>31980</v>
       </c>
       <c r="J615" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K615" s="2" t="inlineStr">
         <is>
@@ -59760,10 +59760,10 @@
         <v>2822</v>
       </c>
       <c r="I618" s="2" t="n">
-        <v>5644</v>
+        <v>8466</v>
       </c>
       <c r="J618" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K618" s="2" t="inlineStr">
         <is>
@@ -59856,10 +59856,10 @@
         <v>2821</v>
       </c>
       <c r="I619" s="2" t="n">
-        <v>31038</v>
+        <v>33859</v>
       </c>
       <c r="J619" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K619" s="2" t="inlineStr">
         <is>
@@ -60144,10 +60144,10 @@
         <v>2730</v>
       </c>
       <c r="I622" s="2" t="n">
-        <v>50009</v>
+        <v>51238</v>
       </c>
       <c r="J622" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K622" s="2" t="inlineStr">
         <is>
@@ -60240,10 +60240,10 @@
         <v>2727</v>
       </c>
       <c r="I623" s="2" t="n">
-        <v>16362</v>
+        <v>19089</v>
       </c>
       <c r="J623" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K623" s="2" t="inlineStr">
         <is>
@@ -60624,10 +60624,10 @@
         <v>2699</v>
       </c>
       <c r="I627" s="2" t="n">
-        <v>10796</v>
+        <v>13495</v>
       </c>
       <c r="J627" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K627" s="2" t="inlineStr">
         <is>
@@ -60720,10 +60720,10 @@
         <v>2698</v>
       </c>
       <c r="I628" s="2" t="n">
-        <v>5396</v>
+        <v>8094</v>
       </c>
       <c r="J628" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K628" s="2" t="inlineStr">
         <is>
@@ -61488,10 +61488,10 @@
         <v>2456</v>
       </c>
       <c r="I636" s="2" t="n">
-        <v>24442</v>
+        <v>26839</v>
       </c>
       <c r="J636" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K636" s="2" t="inlineStr">
         <is>
@@ -61968,10 +61968,10 @@
         <v>2425</v>
       </c>
       <c r="I641" s="2" t="n">
-        <v>20855</v>
+        <v>22795</v>
       </c>
       <c r="J641" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K641" s="2" t="inlineStr">
         <is>
@@ -62160,10 +62160,10 @@
         <v>2355</v>
       </c>
       <c r="I643" s="2" t="n">
-        <v>4710</v>
+        <v>7065</v>
       </c>
       <c r="J643" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K643" s="2" t="inlineStr">
         <is>
@@ -62640,10 +62640,10 @@
         <v>2350</v>
       </c>
       <c r="I648" s="2" t="n">
-        <v>18800</v>
+        <v>21150</v>
       </c>
       <c r="J648" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K648" s="2" t="inlineStr">
         <is>
@@ -62736,10 +62736,10 @@
         <v>2300</v>
       </c>
       <c r="I649" s="2" t="n">
-        <v>4600</v>
+        <v>6900</v>
       </c>
       <c r="J649" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K649" s="2" t="inlineStr">
         <is>
@@ -63024,10 +63024,10 @@
         <v>2249</v>
       </c>
       <c r="I652" s="2" t="n">
-        <v>24107</v>
+        <v>25636</v>
       </c>
       <c r="J652" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K652" s="2" t="inlineStr">
         <is>
@@ -63408,10 +63408,10 @@
         <v>2156</v>
       </c>
       <c r="I656" s="2" t="n">
-        <v>25834</v>
+        <v>27971</v>
       </c>
       <c r="J656" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K656" s="2" t="inlineStr">
         <is>
@@ -63984,10 +63984,10 @@
         <v>2070</v>
       </c>
       <c r="I662" s="2" t="n">
-        <v>4140</v>
+        <v>6210</v>
       </c>
       <c r="J662" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K662" s="2" t="inlineStr">
         <is>
@@ -64368,10 +64368,10 @@
         <v>2014</v>
       </c>
       <c r="I666" s="2" t="n">
-        <v>26255</v>
+        <v>27286</v>
       </c>
       <c r="J666" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K666" s="2" t="inlineStr">
         <is>
@@ -64944,10 +64944,10 @@
         <v>1976</v>
       </c>
       <c r="I672" s="2" t="n">
-        <v>7904</v>
+        <v>9880</v>
       </c>
       <c r="J672" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K672" s="2" t="inlineStr">
         <is>
@@ -65136,10 +65136,10 @@
         <v>1959</v>
       </c>
       <c r="I674" s="2" t="n">
-        <v>3918</v>
+        <v>5877</v>
       </c>
       <c r="J674" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K674" s="2" t="inlineStr">
         <is>
@@ -65232,10 +65232,10 @@
         <v>1953</v>
       </c>
       <c r="I675" s="2" t="n">
-        <v>15626</v>
+        <v>17579</v>
       </c>
       <c r="J675" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K675" s="2" t="inlineStr">
         <is>
@@ -65616,10 +65616,10 @@
         <v>1952</v>
       </c>
       <c r="I679" s="2" t="n">
-        <v>3904</v>
+        <v>5856</v>
       </c>
       <c r="J679" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K679" s="2" t="inlineStr">
         <is>
@@ -65712,10 +65712,10 @@
         <v>1940</v>
       </c>
       <c r="I680" s="2" t="n">
-        <v>32735</v>
+        <v>34675</v>
       </c>
       <c r="J680" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K680" s="2" t="inlineStr">
         <is>
@@ -65904,10 +65904,10 @@
         <v>1929</v>
       </c>
       <c r="I682" s="2" t="n">
-        <v>7716</v>
+        <v>9645</v>
       </c>
       <c r="J682" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K682" s="2" t="inlineStr">
         <is>
@@ -67440,10 +67440,10 @@
         <v>1844</v>
       </c>
       <c r="I698" s="2" t="n">
-        <v>3688</v>
+        <v>5532</v>
       </c>
       <c r="J698" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K698" s="2" t="inlineStr">
         <is>
@@ -67632,10 +67632,10 @@
         <v>1810</v>
       </c>
       <c r="I700" s="2" t="n">
-        <v>5430</v>
+        <v>7240</v>
       </c>
       <c r="J700" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K700" s="2" t="inlineStr">
         <is>
@@ -67920,10 +67920,10 @@
         <v>1799</v>
       </c>
       <c r="I703" s="2" t="n">
-        <v>3598</v>
+        <v>5397</v>
       </c>
       <c r="J703" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K703" s="2" t="inlineStr">
         <is>
@@ -69456,10 +69456,10 @@
         <v>1615</v>
       </c>
       <c r="I719" s="2" t="n">
-        <v>3230</v>
+        <v>4845</v>
       </c>
       <c r="J719" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K719" s="2" t="inlineStr">
         <is>
@@ -69744,10 +69744,10 @@
         <v>1575</v>
       </c>
       <c r="I722" s="2" t="n">
-        <v>9248</v>
+        <v>10722</v>
       </c>
       <c r="J722" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K722" s="2" t="inlineStr">
         <is>
@@ -70224,10 +70224,10 @@
         <v>1524</v>
       </c>
       <c r="I727" s="2" t="n">
-        <v>9144</v>
+        <v>10668</v>
       </c>
       <c r="J727" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K727" s="2" t="inlineStr">
         <is>
@@ -70800,10 +70800,10 @@
         <v>1440</v>
       </c>
       <c r="I733" s="2" t="n">
-        <v>17100</v>
+        <v>18540</v>
       </c>
       <c r="J733" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K733" s="2" t="inlineStr">
         <is>
@@ -71088,10 +71088,10 @@
         <v>1411</v>
       </c>
       <c r="I736" s="2" t="n">
-        <v>5262</v>
+        <v>6673</v>
       </c>
       <c r="J736" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K736" s="2" t="inlineStr">
         <is>
@@ -71280,10 +71280,10 @@
         <v>1411</v>
       </c>
       <c r="I738" s="2" t="n">
-        <v>2822</v>
+        <v>4233</v>
       </c>
       <c r="J738" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K738" s="2" t="inlineStr">
         <is>
@@ -71856,10 +71856,10 @@
         <v>1310</v>
       </c>
       <c r="I744" s="2" t="n">
-        <v>10480</v>
+        <v>11790</v>
       </c>
       <c r="J744" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K744" s="2" t="inlineStr">
         <is>
@@ -72720,10 +72720,10 @@
         <v>1156</v>
       </c>
       <c r="I753" s="2" t="n">
-        <v>8862</v>
+        <v>9913</v>
       </c>
       <c r="J753" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K753" s="2" t="inlineStr">
         <is>
@@ -72816,10 +72816,10 @@
         <v>1128</v>
       </c>
       <c r="I754" s="2" t="n">
-        <v>2256</v>
+        <v>3384</v>
       </c>
       <c r="J754" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K754" s="2" t="inlineStr">
         <is>
@@ -73104,10 +73104,10 @@
         <v>1080</v>
       </c>
       <c r="I757" s="2" t="n">
-        <v>2160</v>
+        <v>3240</v>
       </c>
       <c r="J757" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K757" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(test): isolate test_telegram_sebi_verifier and update 2026-09-13 complete audit reports
</commit_message>
<xml_diff>
--- a/reports/telegram_sebi_10day_report.xlsx
+++ b/reports/telegram_sebi_10day_report.xlsx
@@ -624,10 +624,10 @@
         <v>699669</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>29017536</v>
+        <v>29075144</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -816,10 +816,10 @@
         <v>495829</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>11246216</v>
+        <v>11262987</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -912,10 +912,10 @@
         <v>393135</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>5113173</v>
+        <v>5138197</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -1104,10 +1104,10 @@
         <v>269734</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>6570189</v>
+        <v>6575974</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -1200,10 +1200,10 @@
         <v>222702</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>12867514</v>
+        <v>12870460</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -1296,10 +1296,10 @@
         <v>214868</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>4042130</v>
+        <v>4047926</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1488,10 +1488,10 @@
         <v>211523</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>4512818</v>
+        <v>4517308</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1776,10 +1776,10 @@
         <v>167786</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>3207772</v>
+        <v>3275800</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1872,10 +1872,10 @@
         <v>162819</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>9717252</v>
+        <v>9745156</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -2064,10 +2064,10 @@
         <v>151478</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>6096598</v>
+        <v>6104517</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -2448,10 +2448,10 @@
         <v>136199</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1682933</v>
+        <v>1692684</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
@@ -2544,10 +2544,10 @@
         <v>127846</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>5015169</v>
+        <v>5073836</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -2640,10 +2640,10 @@
         <v>118991</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>5604659</v>
+        <v>5619813</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -3120,10 +3120,10 @@
         <v>106625</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1489642</v>
+        <v>1499578</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -3408,10 +3408,10 @@
         <v>100253</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>3356993</v>
+        <v>3437174</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
@@ -3504,10 +3504,10 @@
         <v>100044</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>1879028</v>
+        <v>1979072</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -3696,10 +3696,10 @@
         <v>99486</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>4361425</v>
+        <v>4397461</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -3888,10 +3888,10 @@
         <v>94432</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>4977569</v>
+        <v>4987391</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -4080,10 +4080,10 @@
         <v>94006</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>2286896</v>
+        <v>2380902</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -4272,10 +4272,10 @@
         <v>92441</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>4713644</v>
+        <v>4727396</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -4464,10 +4464,10 @@
         <v>83780</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>4350330</v>
+        <v>4356646</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -4752,10 +4752,10 @@
         <v>80760</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>1543613</v>
+        <v>1546313</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -5040,10 +5040,10 @@
         <v>79195</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>3393466</v>
+        <v>3402466</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -5136,10 +5136,10 @@
         <v>78907</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>1999585</v>
+        <v>2078492</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
@@ -5328,10 +5328,10 @@
         <v>75133</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>1958358</v>
+        <v>1980934</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -5520,10 +5520,10 @@
         <v>72787</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>2272794</v>
+        <v>2308425</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -5616,10 +5616,10 @@
         <v>72282</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>1545688</v>
+        <v>1570013</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -5712,10 +5712,10 @@
         <v>72252</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>2526069</v>
+        <v>2554917</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -5904,10 +5904,10 @@
         <v>70805</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>4030580</v>
+        <v>4034508</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -6192,10 +6192,10 @@
         <v>69504</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>3441341</v>
+        <v>3469825</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
@@ -6288,10 +6288,10 @@
         <v>68539</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>1673023</v>
+        <v>1677816</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -6480,10 +6480,10 @@
         <v>68202</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>1312343</v>
+        <v>1314130</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
@@ -6576,10 +6576,10 @@
         <v>67494</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>4025145</v>
+        <v>4061738</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
@@ -6672,10 +6672,10 @@
         <v>67038</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>681870</v>
+        <v>748908</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -7152,10 +7152,10 @@
         <v>65111</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>1606077</v>
+        <v>1618135</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
@@ -7248,10 +7248,10 @@
         <v>63293</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>2939899</v>
+        <v>2942340</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
@@ -7344,10 +7344,10 @@
         <v>62414</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>3099796</v>
+        <v>3154621</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
@@ -7440,10 +7440,10 @@
         <v>62347</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>2437039</v>
+        <v>2438593</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
@@ -7920,10 +7920,10 @@
         <v>58524</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>2787249</v>
+        <v>2797041</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
@@ -8016,10 +8016,10 @@
         <v>58230</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>1160201</v>
+        <v>1165054</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
@@ -8400,10 +8400,10 @@
         <v>56909</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>1441051</v>
+        <v>1497960</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
@@ -8592,10 +8592,10 @@
         <v>56639</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>1677412</v>
+        <v>1680122</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
@@ -8688,10 +8688,10 @@
         <v>55901</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>1020182</v>
+        <v>1048132</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
@@ -8784,10 +8784,10 @@
         <v>54547</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>1857693</v>
+        <v>1870351</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
@@ -9072,10 +9072,10 @@
         <v>51138</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>2809738</v>
+        <v>2823405</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -9264,10 +9264,10 @@
         <v>50775</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>2421398</v>
+        <v>2435689</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
@@ -9456,10 +9456,10 @@
         <v>50155</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>2398325</v>
+        <v>2402205</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -9744,10 +9744,10 @@
         <v>49233</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>206779</v>
+        <v>256012</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
@@ -10320,10 +10320,10 @@
         <v>47899</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>1797597</v>
+        <v>1800454</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
@@ -10416,10 +10416,10 @@
         <v>47876</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>1495975</v>
+        <v>1499805</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
@@ -10512,10 +10512,10 @@
         <v>47543</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>1170547</v>
+        <v>1194994</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
@@ -10608,10 +10608,10 @@
         <v>45591</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>1473415</v>
+        <v>1478685</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K106" s="2" t="inlineStr">
         <is>
@@ -10704,10 +10704,10 @@
         <v>45340</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>2562962</v>
+        <v>2566866</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
@@ -11376,10 +11376,10 @@
         <v>41300</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>720919</v>
+        <v>723865</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
@@ -11472,10 +11472,10 @@
         <v>41270</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>1949430</v>
+        <v>1951127</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K115" s="2" t="inlineStr">
         <is>
@@ -11760,10 +11760,10 @@
         <v>40719</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>2042625</v>
+        <v>2043995</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K118" s="2" t="inlineStr">
         <is>
@@ -12048,10 +12048,10 @@
         <v>39193</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>1010615</v>
+        <v>1031191</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K121" s="2" t="inlineStr">
         <is>
@@ -12528,10 +12528,10 @@
         <v>38756</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>2444506</v>
+        <v>2447902</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K126" s="2" t="inlineStr">
         <is>
@@ -12816,10 +12816,10 @@
         <v>38479</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>1449866</v>
+        <v>1459614</v>
       </c>
       <c r="J129" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K129" s="2" t="inlineStr">
         <is>
@@ -13584,10 +13584,10 @@
         <v>36417</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>1411541</v>
+        <v>1416434</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K137" s="2" t="inlineStr">
         <is>
@@ -14064,10 +14064,10 @@
         <v>35379</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>1033713</v>
+        <v>1039084</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
@@ -14544,10 +14544,10 @@
         <v>34556</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>956694</v>
+        <v>960598</v>
       </c>
       <c r="J147" s="2" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K147" s="2" t="inlineStr">
         <is>
@@ -14640,10 +14640,10 @@
         <v>34334</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>1115785</v>
+        <v>1118095</v>
       </c>
       <c r="J148" s="2" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K148" s="2" t="inlineStr">
         <is>
@@ -14736,10 +14736,10 @@
         <v>34011</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>914707</v>
+        <v>919576</v>
       </c>
       <c r="J149" s="2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K149" s="2" t="inlineStr">
         <is>
@@ -15504,10 +15504,10 @@
         <v>33115</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>826118</v>
+        <v>839214</v>
       </c>
       <c r="J157" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
@@ -15600,10 +15600,10 @@
         <v>33063</v>
       </c>
       <c r="I158" s="2" t="n">
-        <v>1745846</v>
+        <v>1748903</v>
       </c>
       <c r="J158" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K158" s="2" t="inlineStr">
         <is>
@@ -15888,10 +15888,10 @@
         <v>32262</v>
       </c>
       <c r="I161" s="2" t="n">
-        <v>943601</v>
+        <v>945293</v>
       </c>
       <c r="J161" s="2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K161" s="2" t="inlineStr">
         <is>
@@ -15984,10 +15984,10 @@
         <v>32087</v>
       </c>
       <c r="I162" s="2" t="n">
-        <v>1536248</v>
+        <v>1539123</v>
       </c>
       <c r="J162" s="2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
@@ -16368,10 +16368,10 @@
         <v>31199</v>
       </c>
       <c r="I166" s="2" t="n">
-        <v>1816242</v>
+        <v>1819849</v>
       </c>
       <c r="J166" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K166" s="2" t="inlineStr">
         <is>
@@ -16464,10 +16464,10 @@
         <v>30867</v>
       </c>
       <c r="I167" s="2" t="n">
-        <v>997848</v>
+        <v>1012229</v>
       </c>
       <c r="J167" s="2" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K167" s="2" t="inlineStr">
         <is>
@@ -16944,10 +16944,10 @@
         <v>29547</v>
       </c>
       <c r="I172" s="2" t="n">
-        <v>1437851</v>
+        <v>1440204</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
@@ -17136,10 +17136,10 @@
         <v>29222</v>
       </c>
       <c r="I174" s="2" t="n">
-        <v>1439855</v>
+        <v>1441772</v>
       </c>
       <c r="J174" s="2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
@@ -17520,10 +17520,10 @@
         <v>28619</v>
       </c>
       <c r="I178" s="2" t="n">
-        <v>471643</v>
+        <v>500262</v>
       </c>
       <c r="J178" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
@@ -17712,10 +17712,10 @@
         <v>28365</v>
       </c>
       <c r="I180" s="2" t="n">
-        <v>1029536</v>
+        <v>1057901</v>
       </c>
       <c r="J180" s="2" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K180" s="2" t="inlineStr">
         <is>
@@ -18384,10 +18384,10 @@
         <v>27294</v>
       </c>
       <c r="I187" s="2" t="n">
-        <v>1285527</v>
+        <v>1297240</v>
       </c>
       <c r="J187" s="2" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K187" s="2" t="inlineStr">
         <is>
@@ -18768,10 +18768,10 @@
         <v>26996</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>931827</v>
+        <v>937652</v>
       </c>
       <c r="J191" s="2" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K191" s="2" t="inlineStr">
         <is>
@@ -19344,10 +19344,10 @@
         <v>26050</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>744296</v>
+        <v>746947</v>
       </c>
       <c r="J197" s="2" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K197" s="2" t="inlineStr">
         <is>
@@ -19440,10 +19440,10 @@
         <v>25641</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>686409</v>
+        <v>692306</v>
       </c>
       <c r="J198" s="2" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K198" s="2" t="inlineStr">
         <is>
@@ -19728,10 +19728,10 @@
         <v>25182</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>635629</v>
+        <v>650010</v>
       </c>
       <c r="J201" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
@@ -19824,10 +19824,10 @@
         <v>25120</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>1208064</v>
+        <v>1210504</v>
       </c>
       <c r="J202" s="2" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
@@ -19920,10 +19920,10 @@
         <v>25014</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>800724</v>
+        <v>802597</v>
       </c>
       <c r="J203" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
@@ -20016,10 +20016,10 @@
         <v>24576</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>788750</v>
+        <v>795101</v>
       </c>
       <c r="J204" s="2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
@@ -20112,10 +20112,10 @@
         <v>24560</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>1326355</v>
+        <v>1333881</v>
       </c>
       <c r="J205" s="2" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K205" s="2" t="inlineStr">
         <is>
@@ -20304,10 +20304,10 @@
         <v>24263</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>291729</v>
+        <v>293281</v>
       </c>
       <c r="J207" s="2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
@@ -20496,10 +20496,10 @@
         <v>23967</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>606805</v>
+        <v>624539</v>
       </c>
       <c r="J209" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
@@ -20976,10 +20976,10 @@
         <v>23148</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>860195</v>
+        <v>865032</v>
       </c>
       <c r="J214" s="2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K214" s="2" t="inlineStr">
         <is>
@@ -21456,10 +21456,10 @@
         <v>22402</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>1517052</v>
+        <v>1535524</v>
       </c>
       <c r="J219" s="2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
@@ -21936,10 +21936,10 @@
         <v>21717</v>
       </c>
       <c r="I224" s="2" t="n">
-        <v>597106</v>
+        <v>606340</v>
       </c>
       <c r="J224" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K224" s="2" t="inlineStr">
         <is>
@@ -22704,10 +22704,10 @@
         <v>21238</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>814576</v>
+        <v>820425</v>
       </c>
       <c r="J232" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K232" s="2" t="inlineStr">
         <is>
@@ -22800,10 +22800,10 @@
         <v>21220</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>244908</v>
+        <v>249223</v>
       </c>
       <c r="J233" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K233" s="2" t="inlineStr">
         <is>
@@ -22896,10 +22896,10 @@
         <v>21217</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>864939</v>
+        <v>868656</v>
       </c>
       <c r="J234" s="2" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K234" s="2" t="inlineStr">
         <is>
@@ -23280,10 +23280,10 @@
         <v>20986</v>
       </c>
       <c r="I238" s="2" t="n">
-        <v>779675</v>
+        <v>800661</v>
       </c>
       <c r="J238" s="2" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K238" s="2" t="inlineStr">
         <is>
@@ -23472,10 +23472,10 @@
         <v>20559</v>
       </c>
       <c r="I240" s="2" t="n">
-        <v>708014</v>
+        <v>725400</v>
       </c>
       <c r="J240" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K240" s="2" t="inlineStr">
         <is>
@@ -23952,10 +23952,10 @@
         <v>20067</v>
       </c>
       <c r="I245" s="2" t="n">
-        <v>861878</v>
+        <v>864333</v>
       </c>
       <c r="J245" s="2" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K245" s="2" t="inlineStr">
         <is>
@@ -24912,10 +24912,10 @@
         <v>19326</v>
       </c>
       <c r="I255" s="2" t="n">
-        <v>782956</v>
+        <v>790235</v>
       </c>
       <c r="J255" s="2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K255" s="2" t="inlineStr">
         <is>
@@ -28080,10 +28080,10 @@
         <v>16494</v>
       </c>
       <c r="I288" s="2" t="n">
-        <v>560021</v>
+        <v>562137</v>
       </c>
       <c r="J288" s="2" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K288" s="2" t="inlineStr">
         <is>
@@ -28272,10 +28272,10 @@
         <v>16436</v>
       </c>
       <c r="I290" s="2" t="n">
-        <v>395379</v>
+        <v>396788</v>
       </c>
       <c r="J290" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K290" s="2" t="inlineStr">
         <is>
@@ -28368,10 +28368,10 @@
         <v>16292</v>
       </c>
       <c r="I291" s="2" t="n">
-        <v>491314</v>
+        <v>493748</v>
       </c>
       <c r="J291" s="2" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K291" s="2" t="inlineStr">
         <is>
@@ -29328,10 +29328,10 @@
         <v>15532</v>
       </c>
       <c r="I301" s="2" t="n">
-        <v>884045</v>
+        <v>894905</v>
       </c>
       <c r="J301" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K301" s="2" t="inlineStr">
         <is>
@@ -29616,10 +29616,10 @@
         <v>15310</v>
       </c>
       <c r="I304" s="2" t="n">
-        <v>796203</v>
+        <v>802003</v>
       </c>
       <c r="J304" s="2" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K304" s="2" t="inlineStr">
         <is>
@@ -29712,10 +29712,10 @@
         <v>15306</v>
       </c>
       <c r="I305" s="2" t="n">
-        <v>472671</v>
+        <v>477940</v>
       </c>
       <c r="J305" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K305" s="2" t="inlineStr">
         <is>
@@ -30384,10 +30384,10 @@
         <v>14767</v>
       </c>
       <c r="I312" s="2" t="n">
-        <v>793185</v>
+        <v>798048</v>
       </c>
       <c r="J312" s="2" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
@@ -30864,10 +30864,10 @@
         <v>14643</v>
       </c>
       <c r="I317" s="2" t="n">
-        <v>413482</v>
+        <v>428007</v>
       </c>
       <c r="J317" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K317" s="2" t="inlineStr">
         <is>
@@ -32208,10 +32208,10 @@
         <v>14114</v>
       </c>
       <c r="I331" s="2" t="n">
-        <v>113379</v>
+        <v>126081</v>
       </c>
       <c r="J331" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
@@ -32304,10 +32304,10 @@
         <v>14114</v>
       </c>
       <c r="I332" s="2" t="n">
-        <v>192514</v>
+        <v>203664</v>
       </c>
       <c r="J332" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K332" s="2" t="inlineStr">
         <is>
@@ -32496,10 +32496,10 @@
         <v>14111</v>
       </c>
       <c r="I334" s="2" t="n">
-        <v>246892</v>
+        <v>260062</v>
       </c>
       <c r="J334" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K334" s="2" t="inlineStr">
         <is>
@@ -32880,10 +32880,10 @@
         <v>13912</v>
       </c>
       <c r="I338" s="2" t="n">
-        <v>373548</v>
+        <v>376249</v>
       </c>
       <c r="J338" s="2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
@@ -33168,10 +33168,10 @@
         <v>13768</v>
       </c>
       <c r="I341" s="2" t="n">
-        <v>347754</v>
+        <v>350273</v>
       </c>
       <c r="J341" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K341" s="2" t="inlineStr">
         <is>
@@ -33360,10 +33360,10 @@
         <v>13645</v>
       </c>
       <c r="I343" s="2" t="n">
-        <v>653084</v>
+        <v>656848</v>
       </c>
       <c r="J343" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K343" s="2" t="inlineStr">
         <is>
@@ -33552,10 +33552,10 @@
         <v>13541</v>
       </c>
       <c r="I345" s="2" t="n">
-        <v>671951</v>
+        <v>676848</v>
       </c>
       <c r="J345" s="2" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K345" s="2" t="inlineStr">
         <is>
@@ -33648,10 +33648,10 @@
         <v>13504</v>
       </c>
       <c r="I346" s="2" t="n">
-        <v>619183</v>
+        <v>625935</v>
       </c>
       <c r="J346" s="2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K346" s="2" t="inlineStr">
         <is>
@@ -33744,10 +33744,10 @@
         <v>13500</v>
       </c>
       <c r="I347" s="2" t="n">
-        <v>451271</v>
+        <v>464771</v>
       </c>
       <c r="J347" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K347" s="2" t="inlineStr">
         <is>
@@ -33840,10 +33840,10 @@
         <v>13500</v>
       </c>
       <c r="I348" s="2" t="n">
-        <v>144014</v>
+        <v>157514</v>
       </c>
       <c r="J348" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K348" s="2" t="inlineStr">
         <is>
@@ -34608,10 +34608,10 @@
         <v>12786</v>
       </c>
       <c r="I356" s="2" t="n">
-        <v>441067</v>
+        <v>443616</v>
       </c>
       <c r="J356" s="2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
@@ -34992,10 +34992,10 @@
         <v>12702</v>
       </c>
       <c r="I360" s="2" t="n">
-        <v>307901</v>
+        <v>312135</v>
       </c>
       <c r="J360" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
@@ -36816,10 +36816,10 @@
         <v>11288</v>
       </c>
       <c r="I379" s="2" t="n">
-        <v>413443</v>
+        <v>415795</v>
       </c>
       <c r="J379" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K379" s="2" t="inlineStr">
         <is>
@@ -37104,10 +37104,10 @@
         <v>11164</v>
       </c>
       <c r="I382" s="2" t="n">
-        <v>286022</v>
+        <v>288978</v>
       </c>
       <c r="J382" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K382" s="2" t="inlineStr">
         <is>
@@ -37200,10 +37200,10 @@
         <v>11161</v>
       </c>
       <c r="I383" s="2" t="n">
-        <v>492530</v>
+        <v>496412</v>
       </c>
       <c r="J383" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K383" s="2" t="inlineStr">
         <is>
@@ -37488,10 +37488,10 @@
         <v>10989</v>
       </c>
       <c r="I386" s="2" t="n">
-        <v>543990</v>
+        <v>548035</v>
       </c>
       <c r="J386" s="2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K386" s="2" t="inlineStr">
         <is>
@@ -37584,10 +37584,10 @@
         <v>10926</v>
       </c>
       <c r="I387" s="2" t="n">
-        <v>363923</v>
+        <v>371233</v>
       </c>
       <c r="J387" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K387" s="2" t="inlineStr">
         <is>
@@ -37680,10 +37680,10 @@
         <v>10833</v>
       </c>
       <c r="I388" s="2" t="n">
-        <v>534954</v>
+        <v>545500</v>
       </c>
       <c r="J388" s="2" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K388" s="2" t="inlineStr">
         <is>
@@ -37872,10 +37872,10 @@
         <v>10726</v>
       </c>
       <c r="I390" s="2" t="n">
-        <v>350488</v>
+        <v>351709</v>
       </c>
       <c r="J390" s="2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K390" s="2" t="inlineStr">
         <is>
@@ -38352,10 +38352,10 @@
         <v>10534</v>
       </c>
       <c r="I395" s="2" t="n">
-        <v>94690</v>
+        <v>105224</v>
       </c>
       <c r="J395" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K395" s="2" t="inlineStr">
         <is>
@@ -39312,10 +39312,10 @@
         <v>10004</v>
       </c>
       <c r="I405" s="2" t="n">
-        <v>106326</v>
+        <v>108136</v>
       </c>
       <c r="J405" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K405" s="2" t="inlineStr">
         <is>
@@ -41424,10 +41424,10 @@
         <v>9587</v>
       </c>
       <c r="I427" s="2" t="n">
-        <v>322875</v>
+        <v>326710</v>
       </c>
       <c r="J427" s="2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K427" s="2" t="inlineStr">
         <is>
@@ -42000,10 +42000,10 @@
         <v>9470</v>
       </c>
       <c r="I433" s="2" t="n">
-        <v>602128</v>
+        <v>604825</v>
       </c>
       <c r="J433" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K433" s="2" t="inlineStr">
         <is>
@@ -42192,10 +42192,10 @@
         <v>9409</v>
       </c>
       <c r="I435" s="2" t="n">
-        <v>238955</v>
+        <v>240366</v>
       </c>
       <c r="J435" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K435" s="2" t="inlineStr">
         <is>
@@ -42480,10 +42480,10 @@
         <v>9306</v>
       </c>
       <c r="I438" s="2" t="n">
-        <v>369930</v>
+        <v>371622</v>
       </c>
       <c r="J438" s="2" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K438" s="2" t="inlineStr">
         <is>
@@ -42768,10 +42768,10 @@
         <v>8999</v>
       </c>
       <c r="I441" s="2" t="n">
-        <v>22045</v>
+        <v>23394</v>
       </c>
       <c r="J441" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K441" s="2" t="inlineStr">
         <is>
@@ -43248,10 +43248,10 @@
         <v>8847</v>
       </c>
       <c r="I446" s="2" t="n">
-        <v>418795</v>
+        <v>420774</v>
       </c>
       <c r="J446" s="2" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K446" s="2" t="inlineStr">
         <is>
@@ -44208,10 +44208,10 @@
         <v>8479</v>
       </c>
       <c r="I456" s="2" t="n">
-        <v>296455</v>
+        <v>299281</v>
       </c>
       <c r="J456" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K456" s="2" t="inlineStr">
         <is>
@@ -44304,10 +44304,10 @@
         <v>8475</v>
       </c>
       <c r="I457" s="2" t="n">
-        <v>590232</v>
+        <v>594977</v>
       </c>
       <c r="J457" s="2" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K457" s="2" t="inlineStr">
         <is>
@@ -44592,10 +44592,10 @@
         <v>8464</v>
       </c>
       <c r="I460" s="2" t="n">
-        <v>314463</v>
+        <v>315874</v>
       </c>
       <c r="J460" s="2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K460" s="2" t="inlineStr">
         <is>
@@ -44784,10 +44784,10 @@
         <v>8363</v>
       </c>
       <c r="I462" s="2" t="n">
-        <v>233179</v>
+        <v>235767</v>
       </c>
       <c r="J462" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K462" s="2" t="inlineStr">
         <is>
@@ -45360,10 +45360,10 @@
         <v>8114</v>
       </c>
       <c r="I468" s="2" t="n">
-        <v>48680</v>
+        <v>56794</v>
       </c>
       <c r="J468" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K468" s="2" t="inlineStr">
         <is>
@@ -46224,10 +46224,10 @@
         <v>7825</v>
       </c>
       <c r="I477" s="2" t="n">
-        <v>422129</v>
+        <v>426034</v>
       </c>
       <c r="J477" s="2" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K477" s="2" t="inlineStr">
         <is>
@@ -47376,10 +47376,10 @@
         <v>7526</v>
       </c>
       <c r="I489" s="2" t="n">
-        <v>67734</v>
+        <v>75260</v>
       </c>
       <c r="J489" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K489" s="2" t="inlineStr">
         <is>
@@ -48912,10 +48912,10 @@
         <v>6890</v>
       </c>
       <c r="I505" s="2" t="n">
-        <v>204636</v>
+        <v>209665</v>
       </c>
       <c r="J505" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K505" s="2" t="inlineStr">
         <is>
@@ -49008,10 +49008,10 @@
         <v>6873</v>
       </c>
       <c r="I506" s="2" t="n">
-        <v>293423</v>
+        <v>300177</v>
       </c>
       <c r="J506" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K506" s="2" t="inlineStr">
         <is>
@@ -49680,10 +49680,10 @@
         <v>6751</v>
       </c>
       <c r="I513" s="2" t="n">
-        <v>347951</v>
+        <v>350744</v>
       </c>
       <c r="J513" s="2" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K513" s="2" t="inlineStr">
         <is>
@@ -50064,10 +50064,10 @@
         <v>6681</v>
       </c>
       <c r="I517" s="2" t="n">
-        <v>191029</v>
+        <v>196205</v>
       </c>
       <c r="J517" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K517" s="2" t="inlineStr">
         <is>
@@ -51024,10 +51024,10 @@
         <v>6529</v>
       </c>
       <c r="I527" s="2" t="n">
-        <v>367139</v>
+        <v>369296</v>
       </c>
       <c r="J527" s="2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K527" s="2" t="inlineStr">
         <is>
@@ -51216,10 +51216,10 @@
         <v>6477</v>
       </c>
       <c r="I529" s="2" t="n">
-        <v>175339</v>
+        <v>177720</v>
       </c>
       <c r="J529" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K529" s="2" t="inlineStr">
         <is>
@@ -52176,10 +52176,10 @@
         <v>6226</v>
       </c>
       <c r="I539" s="2" t="n">
-        <v>61342</v>
+        <v>64482</v>
       </c>
       <c r="J539" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K539" s="2" t="inlineStr">
         <is>
@@ -53520,10 +53520,10 @@
         <v>5857</v>
       </c>
       <c r="I553" s="2" t="n">
-        <v>17571</v>
+        <v>23428</v>
       </c>
       <c r="J553" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K553" s="2" t="inlineStr">
         <is>
@@ -54288,10 +54288,10 @@
         <v>5716</v>
       </c>
       <c r="I561" s="2" t="n">
-        <v>207519</v>
+        <v>212177</v>
       </c>
       <c r="J561" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K561" s="2" t="inlineStr">
         <is>
@@ -55056,10 +55056,10 @@
         <v>5624</v>
       </c>
       <c r="I569" s="2" t="n">
-        <v>155905</v>
+        <v>157650</v>
       </c>
       <c r="J569" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K569" s="2" t="inlineStr">
         <is>
@@ -55536,10 +55536,10 @@
         <v>5420</v>
       </c>
       <c r="I574" s="2" t="n">
-        <v>340227</v>
+        <v>344961</v>
       </c>
       <c r="J574" s="2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K574" s="2" t="inlineStr">
         <is>
@@ -55824,10 +55824,10 @@
         <v>5400</v>
       </c>
       <c r="I577" s="2" t="n">
-        <v>10800</v>
+        <v>16200</v>
       </c>
       <c r="J577" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K577" s="2" t="inlineStr">
         <is>
@@ -56400,10 +56400,10 @@
         <v>5342</v>
       </c>
       <c r="I583" s="2" t="n">
-        <v>166155</v>
+        <v>171497</v>
       </c>
       <c r="J583" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K583" s="2" t="inlineStr">
         <is>
@@ -56976,10 +56976,10 @@
         <v>5206</v>
       </c>
       <c r="I589" s="2" t="n">
-        <v>109128</v>
+        <v>112984</v>
       </c>
       <c r="J589" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K589" s="2" t="inlineStr">
         <is>
@@ -58224,10 +58224,10 @@
         <v>4889</v>
       </c>
       <c r="I602" s="2" t="n">
-        <v>212710</v>
+        <v>217599</v>
       </c>
       <c r="J602" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
@@ -58800,10 +58800,10 @@
         <v>4855</v>
       </c>
       <c r="I608" s="2" t="n">
-        <v>200997</v>
+        <v>204421</v>
       </c>
       <c r="J608" s="2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
@@ -61488,10 +61488,10 @@
         <v>4379</v>
       </c>
       <c r="I636" s="2" t="n">
-        <v>613801</v>
+        <v>617596</v>
       </c>
       <c r="J636" s="2" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K636" s="2" t="inlineStr">
         <is>
@@ -61968,10 +61968,10 @@
         <v>4297</v>
       </c>
       <c r="I641" s="2" t="n">
-        <v>168691</v>
+        <v>170339</v>
       </c>
       <c r="J641" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K641" s="2" t="inlineStr">
         <is>
@@ -62352,10 +62352,10 @@
         <v>4230</v>
       </c>
       <c r="I645" s="2" t="n">
-        <v>141480</v>
+        <v>143460</v>
       </c>
       <c r="J645" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K645" s="2" t="inlineStr">
         <is>
@@ -62448,10 +62448,10 @@
         <v>4155</v>
       </c>
       <c r="I646" s="2" t="n">
-        <v>52676</v>
+        <v>56831</v>
       </c>
       <c r="J646" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K646" s="2" t="inlineStr">
         <is>
@@ -64368,10 +64368,10 @@
         <v>3856</v>
       </c>
       <c r="I666" s="2" t="n">
-        <v>152431</v>
+        <v>153877</v>
       </c>
       <c r="J666" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K666" s="2" t="inlineStr">
         <is>
@@ -65616,10 +65616,10 @@
         <v>3763</v>
       </c>
       <c r="I679" s="2" t="n">
-        <v>40647</v>
+        <v>44410</v>
       </c>
       <c r="J679" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K679" s="2" t="inlineStr">
         <is>
@@ -65808,10 +65808,10 @@
         <v>3762</v>
       </c>
       <c r="I681" s="2" t="n">
-        <v>80418</v>
+        <v>84180</v>
       </c>
       <c r="J681" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K681" s="2" t="inlineStr">
         <is>
@@ -66768,10 +66768,10 @@
         <v>3622</v>
       </c>
       <c r="I691" s="2" t="n">
-        <v>71754</v>
+        <v>73503</v>
       </c>
       <c r="J691" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K691" s="2" t="inlineStr">
         <is>
@@ -67248,10 +67248,10 @@
         <v>3428</v>
       </c>
       <c r="I696" s="2" t="n">
-        <v>119688</v>
+        <v>121402</v>
       </c>
       <c r="J696" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K696" s="2" t="inlineStr">
         <is>
@@ -67632,10 +67632,10 @@
         <v>3405</v>
       </c>
       <c r="I700" s="2" t="n">
-        <v>261308</v>
+        <v>264713</v>
       </c>
       <c r="J700" s="2" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K700" s="2" t="inlineStr">
         <is>
@@ -67824,10 +67824,10 @@
         <v>3392</v>
       </c>
       <c r="I702" s="2" t="n">
-        <v>225776</v>
+        <v>229005</v>
       </c>
       <c r="J702" s="2" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K702" s="2" t="inlineStr">
         <is>
@@ -67920,10 +67920,10 @@
         <v>3387</v>
       </c>
       <c r="I703" s="2" t="n">
-        <v>28981</v>
+        <v>32368</v>
       </c>
       <c r="J703" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K703" s="2" t="inlineStr">
         <is>
@@ -68592,10 +68592,10 @@
         <v>3294</v>
       </c>
       <c r="I710" s="2" t="n">
-        <v>6588</v>
+        <v>9882</v>
       </c>
       <c r="J710" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K710" s="2" t="inlineStr">
         <is>
@@ -69168,10 +69168,10 @@
         <v>3214</v>
       </c>
       <c r="I716" s="2" t="n">
-        <v>118299</v>
+        <v>119615</v>
       </c>
       <c r="J716" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K716" s="2" t="inlineStr">
         <is>
@@ -71184,10 +71184,10 @@
         <v>2898</v>
       </c>
       <c r="I737" s="2" t="n">
-        <v>144914</v>
+        <v>146167</v>
       </c>
       <c r="J737" s="2" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K737" s="2" t="inlineStr">
         <is>
@@ -71280,10 +71280,10 @@
         <v>2894</v>
       </c>
       <c r="I738" s="2" t="n">
-        <v>8682</v>
+        <v>11576</v>
       </c>
       <c r="J738" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K738" s="2" t="inlineStr">
         <is>
@@ -73392,10 +73392,10 @@
         <v>2821</v>
       </c>
       <c r="I760" s="2" t="n">
-        <v>122750</v>
+        <v>124161</v>
       </c>
       <c r="J760" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K760" s="2" t="inlineStr">
         <is>
@@ -73680,10 +73680,10 @@
         <v>2744</v>
       </c>
       <c r="I763" s="2" t="n">
-        <v>82792</v>
+        <v>84013</v>
       </c>
       <c r="J763" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K763" s="2" t="inlineStr">
         <is>
@@ -75312,10 +75312,10 @@
         <v>2441</v>
       </c>
       <c r="I780" s="2" t="n">
-        <v>25390</v>
+        <v>26855</v>
       </c>
       <c r="J780" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K780" s="2" t="inlineStr">
         <is>
@@ -77136,10 +77136,10 @@
         <v>2096</v>
       </c>
       <c r="I799" s="2" t="n">
-        <v>40975</v>
+        <v>42122</v>
       </c>
       <c r="J799" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K799" s="2" t="inlineStr">
         <is>
@@ -77712,10 +77712,10 @@
         <v>2050</v>
       </c>
       <c r="I805" s="2" t="n">
-        <v>32140</v>
+        <v>33860</v>
       </c>
       <c r="J805" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K805" s="2" t="inlineStr">
         <is>
@@ -79344,10 +79344,10 @@
         <v>1937</v>
       </c>
       <c r="I822" s="2" t="n">
-        <v>112770</v>
+        <v>113908</v>
       </c>
       <c r="J822" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K822" s="2" t="inlineStr">
         <is>
@@ -81456,10 +81456,10 @@
         <v>1799</v>
       </c>
       <c r="I844" s="2" t="n">
-        <v>3598</v>
+        <v>5397</v>
       </c>
       <c r="J844" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K844" s="2" t="inlineStr">
         <is>
@@ -81936,10 +81936,10 @@
         <v>1710</v>
       </c>
       <c r="I849" s="2" t="n">
-        <v>46800</v>
+        <v>48510</v>
       </c>
       <c r="J849" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K849" s="2" t="inlineStr">
         <is>
@@ -83088,10 +83088,10 @@
         <v>1591</v>
       </c>
       <c r="I861" s="2" t="n">
-        <v>32532</v>
+        <v>33562</v>
       </c>
       <c r="J861" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K861" s="2" t="inlineStr">
         <is>
@@ -83472,10 +83472,10 @@
         <v>1536</v>
       </c>
       <c r="I865" s="2" t="n">
-        <v>34101</v>
+        <v>35104</v>
       </c>
       <c r="J865" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K865" s="2" t="inlineStr">
         <is>
@@ -84528,10 +84528,10 @@
         <v>1464</v>
       </c>
       <c r="I876" s="2" t="n">
-        <v>2928</v>
+        <v>4392</v>
       </c>
       <c r="J876" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K876" s="2" t="inlineStr">
         <is>
@@ -86064,10 +86064,10 @@
         <v>1279</v>
       </c>
       <c r="I892" s="2" t="n">
-        <v>6170</v>
+        <v>7449</v>
       </c>
       <c r="J892" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K892" s="2" t="inlineStr">
         <is>

</xml_diff>